<commit_message>
Update error handling and add progress tracking
</commit_message>
<xml_diff>
--- a/quality_result.xlsx
+++ b/quality_result.xlsx
@@ -496,37 +496,37 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.007268925030549642</v>
+        <v>0.0850703586590912</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0633366507514582</v>
+        <v>0.8376371584424092</v>
       </c>
       <c r="D2" t="n">
-        <v>0.126950452890563</v>
+        <v>1.664284004585596</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1900679020899734</v>
+        <v>2.517625568475289</v>
       </c>
       <c r="F2" t="n">
-        <v>0.248466219025183</v>
+        <v>3.367084493379861</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3162952418145857</v>
+        <v>4.191526726212222</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3735446402700967</v>
+        <v>5.027392635331763</v>
       </c>
       <c r="I2" t="n">
-        <v>0.4394890336235024</v>
+        <v>5.901832978495572</v>
       </c>
       <c r="J2" t="n">
-        <v>0.5089330931354641</v>
+        <v>6.664221015633858</v>
       </c>
       <c r="K2" t="n">
-        <v>0.5644515551972185</v>
+        <v>6.666145957998967</v>
       </c>
       <c r="L2" t="n">
-        <v>0.6304161050151803</v>
+        <v>6.67339472656496</v>
       </c>
     </row>
     <row r="3">
@@ -536,37 +536,37 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.007268925030549642</v>
+        <v>0.0821375930661762</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0633366507514582</v>
+        <v>0.8415248365436703</v>
       </c>
       <c r="D3" t="n">
-        <v>0.126950452890563</v>
+        <v>1.685579309389133</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1900679020899734</v>
+        <v>2.526804318522531</v>
       </c>
       <c r="F3" t="n">
-        <v>0.248466219025183</v>
+        <v>3.376192695801156</v>
       </c>
       <c r="G3" t="n">
-        <v>0.3162952418145857</v>
+        <v>4.207027047455877</v>
       </c>
       <c r="H3" t="n">
-        <v>0.3735446402700967</v>
+        <v>5.034785018707718</v>
       </c>
       <c r="I3" t="n">
-        <v>0.4394890336235024</v>
+        <v>5.889240227264138</v>
       </c>
       <c r="J3" t="n">
-        <v>0.5089330931354641</v>
+        <v>6.659307877398304</v>
       </c>
       <c r="K3" t="n">
-        <v>0.5644515551972185</v>
+        <v>6.676518978571159</v>
       </c>
       <c r="L3" t="n">
-        <v>0.6304161050151803</v>
+        <v>6.667546832285617</v>
       </c>
     </row>
     <row r="4">
@@ -576,37 +576,37 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.007268925030549642</v>
+        <v>0.0841406417314403</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0633366507514582</v>
+        <v>0.8427493417654544</v>
       </c>
       <c r="D4" t="n">
-        <v>0.126950452890563</v>
+        <v>1.353302510739616</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1900679020899734</v>
+        <v>1.201617556280628</v>
       </c>
       <c r="F4" t="n">
-        <v>0.248466219025183</v>
+        <v>1.711674372315096</v>
       </c>
       <c r="G4" t="n">
-        <v>0.3162120963982917</v>
+        <v>4.184431650688469</v>
       </c>
       <c r="H4" t="n">
-        <v>0.3737411657995188</v>
+        <v>5.034996661585557</v>
       </c>
       <c r="I4" t="n">
-        <v>0.439506670529989</v>
+        <v>4.57409894304539</v>
       </c>
       <c r="J4" t="n">
-        <v>0.508912936670908</v>
+        <v>4.709512591491452</v>
       </c>
       <c r="K4" t="n">
-        <v>0.5645195832650953</v>
+        <v>4.357220423537711</v>
       </c>
       <c r="L4" t="n">
-        <v>0.6310006424873077</v>
+        <v>1.702551052545384</v>
       </c>
     </row>
     <row r="5">
@@ -616,37 +616,37 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.007268925030549642</v>
+        <v>0.0873304022474458</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0633366507514582</v>
+        <v>0.8379672205495157</v>
       </c>
       <c r="D5" t="n">
-        <v>0.126950452890563</v>
+        <v>1.684054976757077</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1900679020899734</v>
+        <v>2.522961992466521</v>
       </c>
       <c r="F5" t="n">
-        <v>0.248466219025183</v>
+        <v>3.336965696216883</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3162952418145857</v>
+        <v>4.207092555965684</v>
       </c>
       <c r="H5" t="n">
-        <v>0.3735446402700967</v>
+        <v>5.036014563045642</v>
       </c>
       <c r="I5" t="n">
-        <v>0.4394890336235024</v>
+        <v>5.895375351163405</v>
       </c>
       <c r="J5" t="n">
-        <v>0.5089330931354641</v>
+        <v>6.673535821816853</v>
       </c>
       <c r="K5" t="n">
-        <v>0.5644515551972185</v>
+        <v>6.660645762733217</v>
       </c>
       <c r="L5" t="n">
-        <v>0.6304161050151803</v>
+        <v>6.673150329432217</v>
       </c>
     </row>
     <row r="6">
@@ -656,37 +656,37 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.007268925030549642</v>
+        <v>0.08590685193817005</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0633366507514582</v>
+        <v>0.8414971214049056</v>
       </c>
       <c r="D6" t="n">
-        <v>0.126950452890563</v>
+        <v>1.684362362841558</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1900679020899734</v>
+        <v>2.523312211038184</v>
       </c>
       <c r="F6" t="n">
-        <v>0.248466219025183</v>
+        <v>3.362957457261996</v>
       </c>
       <c r="G6" t="n">
-        <v>0.3162952418145857</v>
+        <v>4.190919512717469</v>
       </c>
       <c r="H6" t="n">
-        <v>0.3735446402700967</v>
+        <v>5.049045717381171</v>
       </c>
       <c r="I6" t="n">
-        <v>0.4394890336235024</v>
+        <v>5.883928998853601</v>
       </c>
       <c r="J6" t="n">
-        <v>0.5089330931354641</v>
+        <v>6.664452814976253</v>
       </c>
       <c r="K6" t="n">
-        <v>0.5644515551972185</v>
+        <v>6.650156842489827</v>
       </c>
       <c r="L6" t="n">
-        <v>0.6304161050151803</v>
+        <v>6.669018254198214</v>
       </c>
     </row>
     <row r="7">
@@ -696,37 +696,37 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.007268925030549642</v>
+        <v>0.08655941747817433</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0633366507514582</v>
+        <v>0.8423058995452197</v>
       </c>
       <c r="D7" t="n">
-        <v>0.126950452890563</v>
+        <v>1.683523350004409</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1900679020899734</v>
+        <v>2.525761221481752</v>
       </c>
       <c r="F7" t="n">
-        <v>0.248466219025183</v>
+        <v>3.360833469809395</v>
       </c>
       <c r="G7" t="n">
-        <v>0.3162952418145857</v>
+        <v>4.20550523438189</v>
       </c>
       <c r="H7" t="n">
-        <v>0.3735446402700967</v>
+        <v>5.035954093651974</v>
       </c>
       <c r="I7" t="n">
-        <v>0.4394890336235024</v>
+        <v>5.890119553030399</v>
       </c>
       <c r="J7" t="n">
-        <v>0.5089330931354641</v>
+        <v>6.67049219566888</v>
       </c>
       <c r="K7" t="n">
-        <v>0.5644515551972185</v>
+        <v>6.6599528842641</v>
       </c>
       <c r="L7" t="n">
-        <v>0.6304161050151803</v>
+        <v>6.663114929641341</v>
       </c>
     </row>
     <row r="8">
@@ -736,37 +736,37 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.007268925030549642</v>
+        <v>0.08343516547197621</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0633366507514582</v>
+        <v>0.8420438655059902</v>
       </c>
       <c r="D8" t="n">
-        <v>0.126950452890563</v>
+        <v>1.681895715491503</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1900679020899734</v>
+        <v>2.507796772446113</v>
       </c>
       <c r="F8" t="n">
-        <v>0.248466219025183</v>
+        <v>3.357147356353696</v>
       </c>
       <c r="G8" t="n">
-        <v>0.3162952418145857</v>
+        <v>4.198243868025548</v>
       </c>
       <c r="H8" t="n">
-        <v>0.3735446402700967</v>
+        <v>5.042555335794102</v>
       </c>
       <c r="I8" t="n">
-        <v>0.4394890336235024</v>
+        <v>5.866483578780282</v>
       </c>
       <c r="J8" t="n">
-        <v>0.5089330931354641</v>
+        <v>6.646616863402159</v>
       </c>
       <c r="K8" t="n">
-        <v>0.5644515551972185</v>
+        <v>6.674145554869676</v>
       </c>
       <c r="L8" t="n">
-        <v>0.6304161050151803</v>
+        <v>6.673571095629827</v>
       </c>
     </row>
     <row r="9">
@@ -776,37 +776,37 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.007268925030549642</v>
+        <v>0.08295644943876844</v>
       </c>
       <c r="C9" t="n">
-        <v>0.0633366507514582</v>
+        <v>0.8411670592977991</v>
       </c>
       <c r="D9" t="n">
-        <v>0.126950452890563</v>
+        <v>1.670970911702087</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1900679020899734</v>
+        <v>2.519142342433137</v>
       </c>
       <c r="F9" t="n">
-        <v>0.248466219025183</v>
+        <v>3.358865694957105</v>
       </c>
       <c r="G9" t="n">
-        <v>0.3162952418145857</v>
+        <v>4.192972952544124</v>
       </c>
       <c r="H9" t="n">
-        <v>0.3735446402700967</v>
+        <v>5.044694440595119</v>
       </c>
       <c r="I9" t="n">
-        <v>0.4394890336235024</v>
+        <v>5.875443127275476</v>
       </c>
       <c r="J9" t="n">
-        <v>0.5089330931354641</v>
+        <v>6.659267564469192</v>
       </c>
       <c r="K9" t="n">
-        <v>0.5644515551972185</v>
+        <v>6.670421648042933</v>
       </c>
       <c r="L9" t="n">
-        <v>0.6304161050151803</v>
+        <v>6.664336915305055</v>
       </c>
     </row>
     <row r="10">
@@ -816,37 +816,37 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.007268925030549642</v>
+        <v>0.08421118935738671</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0633366507514582</v>
+        <v>0.8440821879842275</v>
       </c>
       <c r="D10" t="n">
-        <v>0.126950452890563</v>
+        <v>1.667410776149863</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1900679020899734</v>
+        <v>2.518522531148037</v>
       </c>
       <c r="F10" t="n">
-        <v>0.248466219025183</v>
+        <v>3.368064601468902</v>
       </c>
       <c r="G10" t="n">
-        <v>0.3162952418145857</v>
+        <v>4.209869108958289</v>
       </c>
       <c r="H10" t="n">
-        <v>0.3735446402700967</v>
+        <v>4.708832310812683</v>
       </c>
       <c r="I10" t="n">
-        <v>0.4394890336235024</v>
+        <v>4.219788609077968</v>
       </c>
       <c r="J10" t="n">
-        <v>0.5089330931354641</v>
+        <v>4.676566850174479</v>
       </c>
       <c r="K10" t="n">
-        <v>0.5644515551972185</v>
+        <v>6.683352020055683</v>
       </c>
       <c r="L10" t="n">
-        <v>0.6304161050151803</v>
+        <v>5.008851207498205</v>
       </c>
     </row>
     <row r="11">
@@ -856,37 +856,37 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.007268925030549642</v>
+        <v>0.08573048287330402</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0633366507514582</v>
+        <v>0.8453772408319581</v>
       </c>
       <c r="D11" t="n">
-        <v>0.126950452890563</v>
+        <v>1.676949823001046</v>
       </c>
       <c r="E11" t="n">
-        <v>0.1900679020899734</v>
+        <v>2.534431020798952</v>
       </c>
       <c r="F11" t="n">
-        <v>0.248466219025183</v>
+        <v>3.357107043424584</v>
       </c>
       <c r="G11" t="n">
-        <v>0.3162952418145857</v>
+        <v>4.191589715163961</v>
       </c>
       <c r="H11" t="n">
-        <v>0.3735446402700967</v>
+        <v>5.03566434447398</v>
       </c>
       <c r="I11" t="n">
-        <v>0.4394890336235024</v>
+        <v>5.862628654933925</v>
       </c>
       <c r="J11" t="n">
-        <v>0.5089330931354641</v>
+        <v>6.654923846357349</v>
       </c>
       <c r="K11" t="n">
-        <v>0.5644515551972185</v>
+        <v>6.679580241625619</v>
       </c>
       <c r="L11" t="n">
-        <v>0.6304161050151803</v>
+        <v>6.655256428022525</v>
       </c>
     </row>
     <row r="12">
@@ -896,37 +896,37 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.007268925030549642</v>
+        <v>0.08471006185515061</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0633366507514582</v>
+        <v>0.8411922548784944</v>
       </c>
       <c r="D12" t="n">
-        <v>0.126950452890563</v>
+        <v>1.682288766550347</v>
       </c>
       <c r="E12" t="n">
-        <v>0.1900679020899734</v>
+        <v>2.518200027715139</v>
       </c>
       <c r="F12" t="n">
-        <v>0.248466219025183</v>
+        <v>3.370558963957722</v>
       </c>
       <c r="G12" t="n">
-        <v>0.3162952418145857</v>
+        <v>4.203779337104272</v>
       </c>
       <c r="H12" t="n">
-        <v>0.3735446402700967</v>
+        <v>5.029541818365058</v>
       </c>
       <c r="I12" t="n">
-        <v>0.4394890336235024</v>
+        <v>5.861026216001713</v>
       </c>
       <c r="J12" t="n">
-        <v>0.5089330931354641</v>
+        <v>6.664596429786216</v>
       </c>
       <c r="K12" t="n">
-        <v>0.5644515551972185</v>
+        <v>6.672454931405031</v>
       </c>
       <c r="L12" t="n">
-        <v>0.6304161050151803</v>
+        <v>6.652081784854937</v>
       </c>
     </row>
     <row r="13">
@@ -936,37 +936,37 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.007268925030549642</v>
+        <v>0.08656445659431336</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0633366507514582</v>
+        <v>0.8373952808677358</v>
       </c>
       <c r="D13" t="n">
-        <v>0.126950452890563</v>
+        <v>1.67427909144736</v>
       </c>
       <c r="E13" t="n">
-        <v>0.1900679020899734</v>
+        <v>2.528772093374822</v>
       </c>
       <c r="F13" t="n">
-        <v>0.248466219025183</v>
+        <v>3.352458458786329</v>
       </c>
       <c r="G13" t="n">
-        <v>0.3162952418145857</v>
+        <v>4.200904521346955</v>
       </c>
       <c r="H13" t="n">
-        <v>0.3735446402700967</v>
+        <v>5.040862192771388</v>
       </c>
       <c r="I13" t="n">
-        <v>0.4394890336235024</v>
+        <v>5.890552917018355</v>
       </c>
       <c r="J13" t="n">
-        <v>0.5089330931354641</v>
+        <v>6.663049421131533</v>
       </c>
       <c r="K13" t="n">
-        <v>0.5644515551972185</v>
+        <v>6.65616346892755</v>
       </c>
       <c r="L13" t="n">
-        <v>0.6304161050151803</v>
+        <v>6.659335592537069</v>
       </c>
     </row>
     <row r="14">
@@ -976,37 +976,37 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.007268925030549642</v>
+        <v>0.08489398959422517</v>
       </c>
       <c r="C14" t="n">
-        <v>0.0633366507514582</v>
+        <v>0.8385593166958516</v>
       </c>
       <c r="D14" t="n">
-        <v>0.126950452890563</v>
+        <v>1.684553849254841</v>
       </c>
       <c r="E14" t="n">
-        <v>0.1900679020899734</v>
+        <v>2.532997392257398</v>
       </c>
       <c r="F14" t="n">
-        <v>0.248466219025183</v>
+        <v>3.363012887539526</v>
       </c>
       <c r="G14" t="n">
-        <v>0.3162952418145857</v>
+        <v>4.199150908930574</v>
       </c>
       <c r="H14" t="n">
-        <v>0.3735446402700967</v>
+        <v>5.048541805767268</v>
       </c>
       <c r="I14" t="n">
-        <v>0.4394890336235024</v>
+        <v>5.881590848965091</v>
       </c>
       <c r="J14" t="n">
-        <v>0.5089330931354641</v>
+        <v>6.689499741745298</v>
       </c>
       <c r="K14" t="n">
-        <v>0.5644515551972185</v>
+        <v>6.656508648383074</v>
       </c>
       <c r="L14" t="n">
-        <v>0.6304161050151803</v>
+        <v>6.660708751684955</v>
       </c>
     </row>
     <row r="15">
@@ -1016,37 +1016,37 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.007268925030549642</v>
+        <v>0.08512074982048148</v>
       </c>
       <c r="C15" t="n">
-        <v>0.0633366507514582</v>
+        <v>0.8384963277441136</v>
       </c>
       <c r="D15" t="n">
-        <v>0.126950452890563</v>
+        <v>1.684478262512755</v>
       </c>
       <c r="E15" t="n">
-        <v>0.1900679020899734</v>
+        <v>2.526925257309868</v>
       </c>
       <c r="F15" t="n">
-        <v>0.248466219025183</v>
+        <v>3.357462301112385</v>
       </c>
       <c r="G15" t="n">
-        <v>0.3162952418145857</v>
+        <v>4.201655349651671</v>
       </c>
       <c r="H15" t="n">
-        <v>0.3735446402700967</v>
+        <v>5.048466219025183</v>
       </c>
       <c r="I15" t="n">
-        <v>0.4394890336235024</v>
+        <v>5.881815089633278</v>
       </c>
       <c r="J15" t="n">
-        <v>0.5089330931354641</v>
+        <v>6.673334257171292</v>
       </c>
       <c r="K15" t="n">
-        <v>0.5644515551972185</v>
+        <v>6.66535229720707</v>
       </c>
       <c r="L15" t="n">
-        <v>0.6304161050151803</v>
+        <v>6.670769347056527</v>
       </c>
     </row>
     <row r="16">
@@ -1056,37 +1056,37 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.007268925030549642</v>
+        <v>0.08478060948109702</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0633366507514582</v>
+        <v>0.8396049332947001</v>
       </c>
       <c r="D16" t="n">
-        <v>0.126950452890563</v>
+        <v>1.668695750765316</v>
       </c>
       <c r="E16" t="n">
-        <v>0.1900679020899734</v>
+        <v>2.520538177603648</v>
       </c>
       <c r="F16" t="n">
-        <v>0.248466219025183</v>
+        <v>3.367346527419091</v>
       </c>
       <c r="G16" t="n">
-        <v>0.3162952418145857</v>
+        <v>4.194930649164137</v>
       </c>
       <c r="H16" t="n">
-        <v>0.3735446402700967</v>
+        <v>5.028191335239799</v>
       </c>
       <c r="I16" t="n">
-        <v>0.4394890336235024</v>
+        <v>5.859942806031822</v>
       </c>
       <c r="J16" t="n">
-        <v>0.5089330931354641</v>
+        <v>6.645233626021995</v>
       </c>
       <c r="K16" t="n">
-        <v>0.5644515551972185</v>
+        <v>6.674069968127591</v>
       </c>
       <c r="L16" t="n">
-        <v>0.6304161050151803</v>
+        <v>6.660466874110281</v>
       </c>
     </row>
   </sheetData>
@@ -1167,37 +1167,37 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>111.6855300245359</v>
+        <v>101.002449283477</v>
       </c>
       <c r="C2" t="n">
-        <v>102.283680980479</v>
+        <v>91.06967257308328</v>
       </c>
       <c r="D2" t="n">
-        <v>99.26388937614198</v>
+        <v>88.08795752952348</v>
       </c>
       <c r="E2" t="n">
-        <v>97.51114411018726</v>
+        <v>86.29032051623656</v>
       </c>
       <c r="F2" t="n">
-        <v>96.34755840888917</v>
+        <v>85.02769177474745</v>
       </c>
       <c r="G2" t="n">
-        <v>95.29930533495903</v>
+        <v>84.07650952481842</v>
       </c>
       <c r="H2" t="n">
-        <v>94.57680682751437</v>
+        <v>83.28680387551285</v>
       </c>
       <c r="I2" t="n">
-        <v>93.87075149368697</v>
+        <v>82.59036277323398</v>
       </c>
       <c r="J2" t="n">
-        <v>93.23362500568271</v>
+        <v>82.06273800352682</v>
       </c>
       <c r="K2" t="n">
-        <v>92.78396518193587</v>
+        <v>82.06148373670189</v>
       </c>
       <c r="L2" t="n">
-        <v>92.30395892765245</v>
+        <v>82.0567637833345</v>
       </c>
     </row>
     <row r="3">
@@ -1207,37 +1207,37 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>111.7055234869341</v>
+        <v>101.1748056611722</v>
       </c>
       <c r="C3" t="n">
-        <v>102.3036744428772</v>
+        <v>91.06955600239758</v>
       </c>
       <c r="D3" t="n">
-        <v>99.28388283854014</v>
+        <v>88.05273346758538</v>
       </c>
       <c r="E3" t="n">
-        <v>97.53113757258544</v>
+        <v>86.29450927925363</v>
       </c>
       <c r="F3" t="n">
-        <v>96.36755187128736</v>
+        <v>85.03595312426867</v>
       </c>
       <c r="G3" t="n">
-        <v>95.31929879735721</v>
+        <v>84.08047234239729</v>
       </c>
       <c r="H3" t="n">
-        <v>94.59680028991255</v>
+        <v>83.30041607135762</v>
       </c>
       <c r="I3" t="n">
-        <v>93.89074495608513</v>
+        <v>82.61963268461295</v>
       </c>
       <c r="J3" t="n">
-        <v>93.25361846808087</v>
+        <v>82.08593444456284</v>
       </c>
       <c r="K3" t="n">
-        <v>92.80395864433405</v>
+        <v>82.07472450535532</v>
       </c>
       <c r="L3" t="n">
-        <v>92.32395239005061</v>
+        <v>82.08056463573995</v>
       </c>
     </row>
     <row r="4">
@@ -1247,37 +1247,37 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>110.9305937711746</v>
+        <v>100.2952374680846</v>
       </c>
       <c r="C4" t="n">
-        <v>101.5287447271177</v>
+        <v>90.28831144833649</v>
       </c>
       <c r="D4" t="n">
-        <v>98.50895312278064</v>
+        <v>88.23134679267397</v>
       </c>
       <c r="E4" t="n">
-        <v>96.75620785682595</v>
+        <v>88.74763301835343</v>
       </c>
       <c r="F4" t="n">
-        <v>95.59262215552789</v>
+        <v>87.2110841848518</v>
       </c>
       <c r="G4" t="n">
-        <v>94.54551087374837</v>
+        <v>83.32893088415524</v>
       </c>
       <c r="H4" t="n">
-        <v>93.81958630876878</v>
+        <v>82.52530379884186</v>
       </c>
       <c r="I4" t="n">
-        <v>93.11564095935636</v>
+        <v>82.94224012154626</v>
       </c>
       <c r="J4" t="n">
-        <v>92.47886075950277</v>
+        <v>82.81553604440928</v>
       </c>
       <c r="K4" t="n">
-        <v>92.02850554558411</v>
+        <v>83.15320036190747</v>
       </c>
       <c r="L4" t="n">
-        <v>91.54499765373731</v>
+        <v>87.23429423322395</v>
       </c>
     </row>
     <row r="5">
@@ -1287,37 +1287,37 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>111.7113417679691</v>
+        <v>100.9143890595644</v>
       </c>
       <c r="C5" t="n">
-        <v>102.3094927239122</v>
+        <v>91.09377336188474</v>
       </c>
       <c r="D5" t="n">
-        <v>99.28970111957511</v>
+        <v>88.0624810135769</v>
       </c>
       <c r="E5" t="n">
-        <v>97.5369558536204</v>
+        <v>86.30693658424363</v>
       </c>
       <c r="F5" t="n">
-        <v>96.37337015232232</v>
+        <v>85.09252624338217</v>
       </c>
       <c r="G5" t="n">
-        <v>95.32511707839218</v>
+        <v>84.08622299904451</v>
       </c>
       <c r="H5" t="n">
-        <v>94.60261857094751</v>
+        <v>83.30517389176177</v>
       </c>
       <c r="I5" t="n">
-        <v>93.89656323712009</v>
+        <v>82.62092905200852</v>
       </c>
       <c r="J5" t="n">
-        <v>93.25943674911585</v>
+        <v>82.08248370507262</v>
       </c>
       <c r="K5" t="n">
-        <v>92.80977692536902</v>
+        <v>82.09088029580408</v>
       </c>
       <c r="L5" t="n">
-        <v>92.32977067108558</v>
+        <v>82.0827345796547</v>
       </c>
     </row>
     <row r="6">
@@ -1327,37 +1327,37 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>111.7057236098203</v>
+        <v>100.9801474610366</v>
       </c>
       <c r="C6" t="n">
-        <v>102.3038745657634</v>
+        <v>91.06989916004068</v>
       </c>
       <c r="D6" t="n">
-        <v>99.28408296142634</v>
+        <v>88.05607022157538</v>
       </c>
       <c r="E6" t="n">
-        <v>97.53133769547163</v>
+        <v>86.30071561305996</v>
       </c>
       <c r="F6" t="n">
-        <v>96.36775199417356</v>
+        <v>85.05321177330062</v>
       </c>
       <c r="G6" t="n">
-        <v>95.31949892024342</v>
+        <v>84.09733230464352</v>
       </c>
       <c r="H6" t="n">
-        <v>94.59700041279874</v>
+        <v>83.28833247581784</v>
       </c>
       <c r="I6" t="n">
-        <v>93.89094507897133</v>
+        <v>82.62375127210797</v>
       </c>
       <c r="J6" t="n">
-        <v>93.25381859096707</v>
+        <v>82.08278053225956</v>
       </c>
       <c r="K6" t="n">
-        <v>92.80415876722024</v>
+        <v>82.09210662519041</v>
       </c>
       <c r="L6" t="n">
-        <v>92.32415251293682</v>
+        <v>82.07980644527389</v>
       </c>
     </row>
     <row r="7">
@@ -1367,37 +1367,37 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>111.7293480511906</v>
+        <v>100.9709066973388</v>
       </c>
       <c r="C7" t="n">
-        <v>102.3274990071336</v>
+        <v>91.08935152301382</v>
       </c>
       <c r="D7" t="n">
-        <v>99.30770740279658</v>
+        <v>88.08185850509486</v>
       </c>
       <c r="E7" t="n">
-        <v>97.55496213684188</v>
+        <v>86.32012703665819</v>
       </c>
       <c r="F7" t="n">
-        <v>96.3913764355438</v>
+        <v>85.07958001224276</v>
       </c>
       <c r="G7" t="n">
-        <v>95.34312336161365</v>
+        <v>84.10586816963516</v>
       </c>
       <c r="H7" t="n">
-        <v>94.62062485416899</v>
+        <v>83.3232323227309</v>
       </c>
       <c r="I7" t="n">
-        <v>93.91456952034159</v>
+        <v>82.64280884974428</v>
       </c>
       <c r="J7" t="n">
-        <v>93.27744303233732</v>
+        <v>82.1024711443022</v>
       </c>
       <c r="K7" t="n">
-        <v>92.8277832085905</v>
+        <v>82.10933838048587</v>
       </c>
       <c r="L7" t="n">
-        <v>92.34777695430708</v>
+        <v>82.10727690500015</v>
       </c>
     </row>
     <row r="8">
@@ -1407,37 +1407,37 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>111.7288999020148</v>
+        <v>101.1301104831033</v>
       </c>
       <c r="C8" t="n">
-        <v>102.3270508579579</v>
+        <v>91.09025463639162</v>
       </c>
       <c r="D8" t="n">
-        <v>99.30725925362086</v>
+        <v>88.0856111566448</v>
       </c>
       <c r="E8" t="n">
-        <v>97.55451398766617</v>
+        <v>86.35067840798538</v>
       </c>
       <c r="F8" t="n">
-        <v>96.39092828636808</v>
+        <v>85.0838977560803</v>
       </c>
       <c r="G8" t="n">
-        <v>95.34267521243794</v>
+        <v>84.11292517580387</v>
       </c>
       <c r="H8" t="n">
-        <v>94.62017670499327</v>
+        <v>83.31709507147899</v>
       </c>
       <c r="I8" t="n">
-        <v>93.91412137116586</v>
+        <v>82.65982320552195</v>
       </c>
       <c r="J8" t="n">
-        <v>93.27699488316159</v>
+        <v>82.11759534813568</v>
       </c>
       <c r="K8" t="n">
-        <v>92.82733505941479</v>
+        <v>82.09964506054241</v>
       </c>
       <c r="L8" t="n">
-        <v>92.34732880513135</v>
+        <v>82.10001888399796</v>
       </c>
     </row>
     <row r="9">
@@ -1447,37 +1447,37 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>111.6676753666291</v>
+        <v>101.0938757052084</v>
       </c>
       <c r="C9" t="n">
-        <v>102.2658263225722</v>
+        <v>91.03355469298357</v>
       </c>
       <c r="D9" t="n">
-        <v>99.24603471823511</v>
+        <v>88.05268836612444</v>
       </c>
       <c r="E9" t="n">
-        <v>97.49328945228042</v>
+        <v>86.2698501865666</v>
       </c>
       <c r="F9" t="n">
-        <v>96.32970375098236</v>
+        <v>85.02045087543083</v>
       </c>
       <c r="G9" t="n">
-        <v>95.28145067705219</v>
+        <v>84.0571566543865</v>
       </c>
       <c r="H9" t="n">
-        <v>94.55895216960754</v>
+        <v>83.2540286040586</v>
       </c>
       <c r="I9" t="n">
-        <v>93.8528968357801</v>
+        <v>82.59197099594884</v>
       </c>
       <c r="J9" t="n">
-        <v>93.21577034777587</v>
+        <v>82.04811261488138</v>
       </c>
       <c r="K9" t="n">
-        <v>92.76611052402902</v>
+        <v>82.0408443912939</v>
       </c>
       <c r="L9" t="n">
-        <v>92.28610426974561</v>
+        <v>82.04480781668741</v>
       </c>
     </row>
     <row r="10">
@@ -1487,37 +1487,37 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>111.2697390554289</v>
+        <v>100.6307429408494</v>
       </c>
       <c r="C10" t="n">
-        <v>101.867890011372</v>
+        <v>90.62059359459155</v>
       </c>
       <c r="D10" t="n">
-        <v>98.8480984070349</v>
+        <v>87.66401491313431</v>
       </c>
       <c r="E10" t="n">
-        <v>97.09535314108021</v>
+        <v>85.87298254757485</v>
       </c>
       <c r="F10" t="n">
-        <v>95.93176743978213</v>
+        <v>84.61063682311604</v>
       </c>
       <c r="G10" t="n">
-        <v>94.88351436585199</v>
+        <v>83.64175502054458</v>
       </c>
       <c r="H10" t="n">
-        <v>94.16101585840732</v>
+        <v>83.15530870459533</v>
       </c>
       <c r="I10" t="n">
-        <v>93.45496052457989</v>
+        <v>83.63153399782277</v>
       </c>
       <c r="J10" t="n">
-        <v>92.81783403657565</v>
+        <v>83.18516948403656</v>
       </c>
       <c r="K10" t="n">
-        <v>92.36817421282882</v>
+        <v>81.63449758713683</v>
       </c>
       <c r="L10" t="n">
-        <v>91.88816795854541</v>
+        <v>82.88705964477124</v>
       </c>
     </row>
     <row r="11">
@@ -1527,37 +1527,37 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>111.7240816165265</v>
+        <v>101.0074308147476</v>
       </c>
       <c r="C11" t="n">
-        <v>102.3222325724696</v>
+        <v>91.06827799739176</v>
       </c>
       <c r="D11" t="n">
-        <v>99.30244096813252</v>
+        <v>88.09358283332958</v>
       </c>
       <c r="E11" t="n">
-        <v>97.54969570217779</v>
+        <v>86.29997875756328</v>
       </c>
       <c r="F11" t="n">
-        <v>96.38611000087971</v>
+        <v>85.07913162137926</v>
       </c>
       <c r="G11" t="n">
-        <v>95.33785692694957</v>
+        <v>84.11499585288388</v>
       </c>
       <c r="H11" t="n">
-        <v>94.61535841950491</v>
+        <v>83.3182157713799</v>
       </c>
       <c r="I11" t="n">
-        <v>93.90930308567749</v>
+        <v>82.65785964966963</v>
       </c>
       <c r="J11" t="n">
-        <v>93.27217659767325</v>
+        <v>82.10735261234274</v>
       </c>
       <c r="K11" t="n">
-        <v>92.8225167739264</v>
+        <v>82.09129179966925</v>
       </c>
       <c r="L11" t="n">
-        <v>92.34251051964299</v>
+        <v>82.10713557789389</v>
       </c>
     </row>
     <row r="12">
@@ -1567,37 +1567,37 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>111.7010930471644</v>
+        <v>101.0364449555497</v>
       </c>
       <c r="C12" t="n">
-        <v>102.2992440031075</v>
+        <v>91.06684229070513</v>
       </c>
       <c r="D12" t="n">
-        <v>99.27945239877042</v>
+        <v>88.05678949474287</v>
       </c>
       <c r="E12" t="n">
-        <v>97.52670713281572</v>
+        <v>86.30489270042447</v>
       </c>
       <c r="F12" t="n">
-        <v>96.36312143151763</v>
+        <v>85.03877565405878</v>
       </c>
       <c r="G12" t="n">
-        <v>95.31486835758749</v>
+        <v>84.07939583253662</v>
       </c>
       <c r="H12" t="n">
-        <v>94.59236985014283</v>
+        <v>83.30051070955724</v>
       </c>
       <c r="I12" t="n">
-        <v>93.88631451631541</v>
+        <v>82.63605830459525</v>
       </c>
       <c r="J12" t="n">
-        <v>93.24918802831115</v>
+        <v>82.07805638285438</v>
       </c>
       <c r="K12" t="n">
-        <v>92.79952820456433</v>
+        <v>82.07293845357358</v>
       </c>
       <c r="L12" t="n">
-        <v>92.31952195028089</v>
+        <v>82.08621914349041</v>
       </c>
     </row>
     <row r="13">
@@ -1607,37 +1607,37 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>111.71668982828</v>
+        <v>100.9579956542617</v>
       </c>
       <c r="C13" t="n">
-        <v>102.3148407842231</v>
+        <v>91.10208663428818</v>
       </c>
       <c r="D13" t="n">
-        <v>99.29504917988601</v>
+        <v>88.09311318768556</v>
       </c>
       <c r="E13" t="n">
-        <v>97.54230391393131</v>
+        <v>86.30229482389697</v>
       </c>
       <c r="F13" t="n">
-        <v>96.37871821263323</v>
+        <v>85.07775767431613</v>
       </c>
       <c r="G13" t="n">
-        <v>95.33046513870309</v>
+        <v>84.09796361574962</v>
       </c>
       <c r="H13" t="n">
-        <v>94.60796663125841</v>
+        <v>83.30634347682957</v>
       </c>
       <c r="I13" t="n">
-        <v>93.901911297431</v>
+        <v>82.62983110757168</v>
       </c>
       <c r="J13" t="n">
-        <v>93.26478480942674</v>
+        <v>82.09466138002361</v>
       </c>
       <c r="K13" t="n">
-        <v>92.81512498567993</v>
+        <v>82.09915193263504</v>
       </c>
       <c r="L13" t="n">
-        <v>92.33511873139649</v>
+        <v>82.09708271119734</v>
       </c>
     </row>
     <row r="14">
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>111.6866138767071</v>
+        <v>101.0125463363493</v>
       </c>
       <c r="C14" t="n">
-        <v>102.2847648326501</v>
+        <v>91.06597788899977</v>
       </c>
       <c r="D14" t="n">
-        <v>99.26497322831308</v>
+        <v>88.03646678967296</v>
       </c>
       <c r="E14" t="n">
-        <v>97.51222796235837</v>
+        <v>86.26496834690789</v>
       </c>
       <c r="F14" t="n">
-        <v>96.34864226106031</v>
+        <v>85.03403045776155</v>
       </c>
       <c r="G14" t="n">
-        <v>95.30038918713015</v>
+        <v>84.06970094794181</v>
       </c>
       <c r="H14" t="n">
-        <v>94.57789067968548</v>
+        <v>83.26965620472305</v>
       </c>
       <c r="I14" t="n">
-        <v>93.87183534585807</v>
+        <v>82.60636767710155</v>
       </c>
       <c r="J14" t="n">
-        <v>93.23470885785382</v>
+        <v>82.04737936064672</v>
       </c>
       <c r="K14" t="n">
-        <v>92.78504903410699</v>
+        <v>82.06885076777432</v>
       </c>
       <c r="L14" t="n">
-        <v>92.30504277982357</v>
+        <v>82.06611133401256</v>
       </c>
     </row>
     <row r="15">
@@ -1687,37 +1687,37 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>111.6403303307907</v>
+        <v>100.9546778215397</v>
       </c>
       <c r="C15" t="n">
-        <v>102.2384812867338</v>
+        <v>91.02002057858152</v>
       </c>
       <c r="D15" t="n">
-        <v>99.21868968239673</v>
+        <v>87.99037811815325</v>
       </c>
       <c r="E15" t="n">
-        <v>97.46594441644204</v>
+        <v>86.22910826454871</v>
       </c>
       <c r="F15" t="n">
-        <v>96.30235871514398</v>
+        <v>84.99492077838617</v>
       </c>
       <c r="G15" t="n">
-        <v>95.25410564121384</v>
+        <v>84.02082797242988</v>
       </c>
       <c r="H15" t="n">
-        <v>94.53160713376916</v>
+        <v>83.22343768184109</v>
       </c>
       <c r="I15" t="n">
-        <v>93.82555179994172</v>
+        <v>82.55991855586574</v>
       </c>
       <c r="J15" t="n">
-        <v>93.18842531193749</v>
+        <v>82.01160344233861</v>
       </c>
       <c r="K15" t="n">
-        <v>92.73876548819067</v>
+        <v>82.01680113787914</v>
       </c>
       <c r="L15" t="n">
-        <v>92.25875923390724</v>
+        <v>82.01327298321775</v>
       </c>
     </row>
     <row r="16">
@@ -1727,37 +1727,37 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>111.6472635371152</v>
+        <v>100.9790000906037</v>
       </c>
       <c r="C16" t="n">
-        <v>102.2454144930583</v>
+        <v>91.0212156169605</v>
       </c>
       <c r="D16" t="n">
-        <v>99.2256228887212</v>
+        <v>88.03819383371234</v>
       </c>
       <c r="E16" t="n">
-        <v>97.4728776227665</v>
+        <v>86.24703263500228</v>
       </c>
       <c r="F16" t="n">
-        <v>96.30929192146844</v>
+        <v>84.98908732280671</v>
       </c>
       <c r="G16" t="n">
-        <v>95.26103884753829</v>
+        <v>84.03471757969879</v>
       </c>
       <c r="H16" t="n">
-        <v>94.53854034009362</v>
+        <v>83.24784748094297</v>
       </c>
       <c r="I16" t="n">
-        <v>93.8324850062662</v>
+        <v>82.58303166156502</v>
       </c>
       <c r="J16" t="n">
-        <v>93.19535851826195</v>
+        <v>82.03686289404064</v>
       </c>
       <c r="K16" t="n">
-        <v>92.74569869451513</v>
+        <v>82.0180578811012</v>
       </c>
       <c r="L16" t="n">
-        <v>92.2656924402317</v>
+        <v>82.02691870737181</v>
       </c>
     </row>
   </sheetData>
@@ -1838,37 +1838,37 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>117.7147641782954</v>
+        <v>107.0316834372365</v>
       </c>
       <c r="C2" t="n">
-        <v>108.3129151342385</v>
+        <v>97.09890672684276</v>
       </c>
       <c r="D2" t="n">
-        <v>105.2931235299014</v>
+        <v>94.11719168328293</v>
       </c>
       <c r="E2" t="n">
-        <v>103.5403782639467</v>
+        <v>92.31955466999602</v>
       </c>
       <c r="F2" t="n">
-        <v>102.3767925626486</v>
+        <v>91.05692592850693</v>
       </c>
       <c r="G2" t="n">
-        <v>101.3285394887185</v>
+        <v>90.10574367857787</v>
       </c>
       <c r="H2" t="n">
-        <v>100.6060409812738</v>
+        <v>89.31603802927229</v>
       </c>
       <c r="I2" t="n">
-        <v>99.89998564744641</v>
+        <v>88.61959692699344</v>
       </c>
       <c r="J2" t="n">
-        <v>99.26285915944217</v>
+        <v>88.09197215728629</v>
       </c>
       <c r="K2" t="n">
-        <v>98.81319933569534</v>
+        <v>88.09071789046135</v>
       </c>
       <c r="L2" t="n">
-        <v>98.33319308141191</v>
+        <v>88.08599793709396</v>
       </c>
     </row>
     <row r="3">
@@ -1878,37 +1878,37 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>117.7147641782954</v>
+        <v>107.1840463525335</v>
       </c>
       <c r="C3" t="n">
-        <v>108.3129151342385</v>
+        <v>97.07879669375886</v>
       </c>
       <c r="D3" t="n">
-        <v>105.2931235299014</v>
+        <v>94.06197415894668</v>
       </c>
       <c r="E3" t="n">
-        <v>103.5403782639467</v>
+        <v>92.3037499706149</v>
       </c>
       <c r="F3" t="n">
-        <v>102.3767925626486</v>
+        <v>91.04519381562996</v>
       </c>
       <c r="G3" t="n">
-        <v>101.3285394887185</v>
+        <v>90.08971303375857</v>
       </c>
       <c r="H3" t="n">
-        <v>100.6060409812738</v>
+        <v>89.3096567627189</v>
       </c>
       <c r="I3" t="n">
-        <v>99.89998564744641</v>
+        <v>88.62887337597425</v>
       </c>
       <c r="J3" t="n">
-        <v>99.26285915944217</v>
+        <v>88.09517513592412</v>
       </c>
       <c r="K3" t="n">
-        <v>98.81319933569534</v>
+        <v>88.0839651967166</v>
       </c>
       <c r="L3" t="n">
-        <v>98.33319308141191</v>
+        <v>88.08980532710123</v>
       </c>
     </row>
     <row r="4">
@@ -1918,37 +1918,37 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>117.7147641782954</v>
+        <v>107.0794078752054</v>
       </c>
       <c r="C4" t="n">
-        <v>108.3129151342385</v>
+        <v>97.07248185545726</v>
       </c>
       <c r="D4" t="n">
-        <v>105.2931235299014</v>
+        <v>95.01551719979476</v>
       </c>
       <c r="E4" t="n">
-        <v>103.5403782639467</v>
+        <v>95.53180342547419</v>
       </c>
       <c r="F4" t="n">
-        <v>102.3767925626486</v>
+        <v>93.99525459197258</v>
       </c>
       <c r="G4" t="n">
-        <v>101.3296812808692</v>
+        <v>90.11310129127601</v>
       </c>
       <c r="H4" t="n">
-        <v>100.6037567158895</v>
+        <v>89.30947420596266</v>
       </c>
       <c r="I4" t="n">
-        <v>99.89981136647714</v>
+        <v>89.72641052866705</v>
       </c>
       <c r="J4" t="n">
-        <v>99.26303116662353</v>
+        <v>89.59970645153005</v>
       </c>
       <c r="K4" t="n">
-        <v>98.81267595270488</v>
+        <v>89.93737076902823</v>
       </c>
       <c r="L4" t="n">
-        <v>98.32916806085808</v>
+        <v>94.01846464034472</v>
       </c>
     </row>
     <row r="5">
@@ -1958,37 +1958,37 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>117.7147641782954</v>
+        <v>106.9178114698907</v>
       </c>
       <c r="C5" t="n">
-        <v>108.3129151342385</v>
+        <v>97.09719577221107</v>
       </c>
       <c r="D5" t="n">
-        <v>105.2931235299014</v>
+        <v>94.06590342390322</v>
       </c>
       <c r="E5" t="n">
-        <v>103.5403782639467</v>
+        <v>92.31035899456997</v>
       </c>
       <c r="F5" t="n">
-        <v>102.3767925626486</v>
+        <v>91.09594865370849</v>
       </c>
       <c r="G5" t="n">
-        <v>101.3285394887185</v>
+        <v>90.08964540937083</v>
       </c>
       <c r="H5" t="n">
-        <v>100.6060409812738</v>
+        <v>89.30859630208808</v>
       </c>
       <c r="I5" t="n">
-        <v>99.89998564744641</v>
+        <v>88.62435146233483</v>
       </c>
       <c r="J5" t="n">
-        <v>99.26285915944217</v>
+        <v>88.08590611539893</v>
       </c>
       <c r="K5" t="n">
-        <v>98.81319933569534</v>
+        <v>88.09430270613041</v>
       </c>
       <c r="L5" t="n">
-        <v>98.33319308141191</v>
+        <v>88.08615698998102</v>
       </c>
     </row>
     <row r="6">
@@ -1998,37 +1998,37 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>117.7147641782954</v>
+        <v>106.9891880295116</v>
       </c>
       <c r="C6" t="n">
-        <v>108.3129151342385</v>
+        <v>97.07893972851578</v>
       </c>
       <c r="D6" t="n">
-        <v>105.2931235299014</v>
+        <v>94.0651107900505</v>
       </c>
       <c r="E6" t="n">
-        <v>103.5403782639467</v>
+        <v>92.30975618153505</v>
       </c>
       <c r="F6" t="n">
-        <v>102.3767925626486</v>
+        <v>91.06225234177572</v>
       </c>
       <c r="G6" t="n">
-        <v>101.3285394887185</v>
+        <v>90.10637287311859</v>
       </c>
       <c r="H6" t="n">
-        <v>100.6060409812738</v>
+        <v>89.29737304429293</v>
       </c>
       <c r="I6" t="n">
-        <v>99.89998564744641</v>
+        <v>88.63279184058305</v>
       </c>
       <c r="J6" t="n">
-        <v>99.26285915944217</v>
+        <v>88.09182110073468</v>
       </c>
       <c r="K6" t="n">
-        <v>98.81319933569534</v>
+        <v>88.10114719366551</v>
       </c>
       <c r="L6" t="n">
-        <v>98.33319308141191</v>
+        <v>88.08884701374899</v>
       </c>
     </row>
     <row r="7">
@@ -2038,37 +2038,37 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>117.7147641782954</v>
+        <v>106.9563228244436</v>
       </c>
       <c r="C7" t="n">
-        <v>108.3129151342385</v>
+        <v>97.07476765011864</v>
       </c>
       <c r="D7" t="n">
-        <v>105.2931235299014</v>
+        <v>94.06727463219968</v>
       </c>
       <c r="E7" t="n">
-        <v>103.5403782639467</v>
+        <v>92.30554316376302</v>
       </c>
       <c r="F7" t="n">
-        <v>102.3767925626486</v>
+        <v>91.0649961393476</v>
       </c>
       <c r="G7" t="n">
-        <v>101.3285394887185</v>
+        <v>90.09128429674</v>
       </c>
       <c r="H7" t="n">
-        <v>100.6060409812738</v>
+        <v>89.30864844983574</v>
       </c>
       <c r="I7" t="n">
-        <v>99.89998564744641</v>
+        <v>88.62822497684914</v>
       </c>
       <c r="J7" t="n">
-        <v>99.26285915944217</v>
+        <v>88.08788727140706</v>
       </c>
       <c r="K7" t="n">
-        <v>98.81319933569534</v>
+        <v>88.09475450759069</v>
       </c>
       <c r="L7" t="n">
-        <v>98.33319308141191</v>
+        <v>88.09269303210499</v>
       </c>
     </row>
     <row r="8">
@@ -2078,37 +2078,37 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>117.7147641782954</v>
+        <v>107.1159747593838</v>
       </c>
       <c r="C8" t="n">
-        <v>108.3129151342385</v>
+        <v>97.07611891267217</v>
       </c>
       <c r="D8" t="n">
-        <v>105.2931235299014</v>
+        <v>94.07147543292535</v>
       </c>
       <c r="E8" t="n">
-        <v>103.5403782639467</v>
+        <v>92.33654268426592</v>
       </c>
       <c r="F8" t="n">
-        <v>102.3767925626486</v>
+        <v>91.06976203236087</v>
       </c>
       <c r="G8" t="n">
-        <v>101.3285394887185</v>
+        <v>90.09878945208443</v>
       </c>
       <c r="H8" t="n">
-        <v>100.6060409812738</v>
+        <v>89.30295934775954</v>
       </c>
       <c r="I8" t="n">
-        <v>99.89998564744641</v>
+        <v>88.64568748180248</v>
       </c>
       <c r="J8" t="n">
-        <v>99.26285915944217</v>
+        <v>88.10345962441623</v>
       </c>
       <c r="K8" t="n">
-        <v>98.81319933569534</v>
+        <v>88.08550933682297</v>
       </c>
       <c r="L8" t="n">
-        <v>98.33319308141191</v>
+        <v>88.08588316027851</v>
       </c>
     </row>
     <row r="9">
@@ -2118,37 +2118,37 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>117.7147641782954</v>
+        <v>107.1409645168747</v>
       </c>
       <c r="C9" t="n">
-        <v>108.3129151342385</v>
+        <v>97.08064350464987</v>
       </c>
       <c r="D9" t="n">
-        <v>105.2931235299014</v>
+        <v>94.09977717779074</v>
       </c>
       <c r="E9" t="n">
-        <v>103.5403782639467</v>
+        <v>92.3169389982329</v>
       </c>
       <c r="F9" t="n">
-        <v>102.3767925626486</v>
+        <v>91.06753968709712</v>
       </c>
       <c r="G9" t="n">
-        <v>101.3285394887185</v>
+        <v>90.1042454660528</v>
       </c>
       <c r="H9" t="n">
-        <v>100.6060409812738</v>
+        <v>89.30111741572492</v>
       </c>
       <c r="I9" t="n">
-        <v>99.89998564744641</v>
+        <v>88.63905980761515</v>
       </c>
       <c r="J9" t="n">
-        <v>99.26285915944217</v>
+        <v>88.09520142654767</v>
       </c>
       <c r="K9" t="n">
-        <v>98.81319933569534</v>
+        <v>88.08793320296019</v>
       </c>
       <c r="L9" t="n">
-        <v>98.33319308141191</v>
+        <v>88.09189662835372</v>
       </c>
     </row>
     <row r="10">
@@ -2158,37 +2158,37 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>117.7147641782954</v>
+        <v>107.0757680637159</v>
       </c>
       <c r="C10" t="n">
-        <v>108.3129151342385</v>
+        <v>97.06561871745807</v>
       </c>
       <c r="D10" t="n">
-        <v>105.2931235299014</v>
+        <v>94.10904003600082</v>
       </c>
       <c r="E10" t="n">
-        <v>103.5403782639467</v>
+        <v>92.31800767044136</v>
       </c>
       <c r="F10" t="n">
-        <v>102.3767925626486</v>
+        <v>91.05566194598255</v>
       </c>
       <c r="G10" t="n">
-        <v>101.3285394887185</v>
+        <v>90.08678014341112</v>
       </c>
       <c r="H10" t="n">
-        <v>100.6060409812738</v>
+        <v>89.60033382746187</v>
       </c>
       <c r="I10" t="n">
-        <v>99.89998564744641</v>
+        <v>90.07655912068928</v>
       </c>
       <c r="J10" t="n">
-        <v>99.26285915944217</v>
+        <v>89.63019460690307</v>
       </c>
       <c r="K10" t="n">
-        <v>98.81319933569534</v>
+        <v>88.07952271000335</v>
       </c>
       <c r="L10" t="n">
-        <v>98.33319308141191</v>
+        <v>89.33208476763775</v>
       </c>
     </row>
     <row r="11">
@@ -2198,37 +2198,37 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>117.7147641782954</v>
+        <v>106.9981133765165</v>
       </c>
       <c r="C11" t="n">
-        <v>108.3129151342385</v>
+        <v>97.05896055916068</v>
       </c>
       <c r="D11" t="n">
-        <v>105.2931235299014</v>
+        <v>94.0842653950985</v>
       </c>
       <c r="E11" t="n">
-        <v>103.5403782639467</v>
+        <v>92.2906613193322</v>
       </c>
       <c r="F11" t="n">
-        <v>102.3767925626486</v>
+        <v>91.06981418314818</v>
       </c>
       <c r="G11" t="n">
-        <v>101.3285394887185</v>
+        <v>90.10567841465281</v>
       </c>
       <c r="H11" t="n">
-        <v>100.6060409812738</v>
+        <v>89.30889833314882</v>
       </c>
       <c r="I11" t="n">
-        <v>99.89998564744641</v>
+        <v>88.64854221143855</v>
       </c>
       <c r="J11" t="n">
-        <v>99.26285915944217</v>
+        <v>88.09803517411167</v>
       </c>
       <c r="K11" t="n">
-        <v>98.81319933569534</v>
+        <v>88.08197436143817</v>
       </c>
       <c r="L11" t="n">
-        <v>98.33319308141191</v>
+        <v>88.09781813966282</v>
       </c>
     </row>
     <row r="12">
@@ -2238,37 +2238,37 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>117.7147641782954</v>
+        <v>107.0501160866807</v>
       </c>
       <c r="C12" t="n">
-        <v>108.3129151342385</v>
+        <v>97.08051342183614</v>
       </c>
       <c r="D12" t="n">
-        <v>105.2931235299014</v>
+        <v>94.07046062587389</v>
       </c>
       <c r="E12" t="n">
-        <v>103.5403782639467</v>
+        <v>92.31856383155548</v>
       </c>
       <c r="F12" t="n">
-        <v>102.3767925626486</v>
+        <v>91.05244678518979</v>
       </c>
       <c r="G12" t="n">
-        <v>101.3285394887185</v>
+        <v>90.09306696366762</v>
       </c>
       <c r="H12" t="n">
-        <v>100.6060409812738</v>
+        <v>89.31418184068825</v>
       </c>
       <c r="I12" t="n">
-        <v>99.89998564744641</v>
+        <v>88.64972943572626</v>
       </c>
       <c r="J12" t="n">
-        <v>99.26285915944217</v>
+        <v>88.0917275139854</v>
       </c>
       <c r="K12" t="n">
-        <v>98.81319933569534</v>
+        <v>88.0866095847046</v>
       </c>
       <c r="L12" t="n">
-        <v>98.33319308141191</v>
+        <v>88.09989027462143</v>
       </c>
     </row>
     <row r="13">
@@ -2278,37 +2278,37 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>117.7147641782954</v>
+        <v>106.9560700042771</v>
       </c>
       <c r="C13" t="n">
-        <v>108.3129151342385</v>
+        <v>97.10016098430359</v>
       </c>
       <c r="D13" t="n">
-        <v>105.2931235299014</v>
+        <v>94.09118753770096</v>
       </c>
       <c r="E13" t="n">
-        <v>103.5403782639467</v>
+        <v>92.30036917391239</v>
       </c>
       <c r="F13" t="n">
-        <v>102.3767925626486</v>
+        <v>91.07583202433155</v>
       </c>
       <c r="G13" t="n">
-        <v>101.3285394887185</v>
+        <v>90.09603796576505</v>
       </c>
       <c r="H13" t="n">
-        <v>100.6060409812738</v>
+        <v>89.30441782684497</v>
       </c>
       <c r="I13" t="n">
-        <v>99.89998564744641</v>
+        <v>88.62790545758708</v>
       </c>
       <c r="J13" t="n">
-        <v>99.26285915944217</v>
+        <v>88.09273573003904</v>
       </c>
       <c r="K13" t="n">
-        <v>98.81319933569534</v>
+        <v>88.09722628265047</v>
       </c>
       <c r="L13" t="n">
-        <v>98.33319308141191</v>
+        <v>88.09515706121275</v>
       </c>
     </row>
     <row r="14">
@@ -2318,37 +2318,37 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>117.7147641782954</v>
+        <v>107.0406966379376</v>
       </c>
       <c r="C14" t="n">
-        <v>108.3129151342385</v>
+        <v>97.09412819058812</v>
       </c>
       <c r="D14" t="n">
-        <v>105.2931235299014</v>
+        <v>94.06461709126131</v>
       </c>
       <c r="E14" t="n">
-        <v>103.5403782639467</v>
+        <v>92.29311864849626</v>
       </c>
       <c r="F14" t="n">
-        <v>102.3767925626486</v>
+        <v>91.06218075934989</v>
       </c>
       <c r="G14" t="n">
-        <v>101.3285394887185</v>
+        <v>90.09785124953018</v>
       </c>
       <c r="H14" t="n">
-        <v>100.6060409812738</v>
+        <v>89.29780650631137</v>
       </c>
       <c r="I14" t="n">
-        <v>99.89998564744641</v>
+        <v>88.63451797868991</v>
       </c>
       <c r="J14" t="n">
-        <v>99.26285915944217</v>
+        <v>88.07552966223506</v>
       </c>
       <c r="K14" t="n">
-        <v>98.81319933569534</v>
+        <v>88.09700106936268</v>
       </c>
       <c r="L14" t="n">
-        <v>98.33319308141191</v>
+        <v>88.09426163560093</v>
       </c>
     </row>
     <row r="15">
@@ -2358,37 +2358,37 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>117.7147641782954</v>
+        <v>107.0291116690444</v>
       </c>
       <c r="C15" t="n">
-        <v>108.3129151342385</v>
+        <v>97.0944544260862</v>
       </c>
       <c r="D15" t="n">
-        <v>105.2931235299014</v>
+        <v>94.06481196565792</v>
       </c>
       <c r="E15" t="n">
-        <v>103.5403782639467</v>
+        <v>92.30354211205339</v>
       </c>
       <c r="F15" t="n">
-        <v>102.3767925626486</v>
+        <v>91.06935462589085</v>
       </c>
       <c r="G15" t="n">
-        <v>101.3285394887185</v>
+        <v>90.09526181993456</v>
       </c>
       <c r="H15" t="n">
-        <v>100.6060409812738</v>
+        <v>89.29787152934574</v>
       </c>
       <c r="I15" t="n">
-        <v>99.89998564744641</v>
+        <v>88.63435240337041</v>
       </c>
       <c r="J15" t="n">
-        <v>99.26285915944217</v>
+        <v>88.08603728984329</v>
       </c>
       <c r="K15" t="n">
-        <v>98.81319933569534</v>
+        <v>88.09123498538382</v>
       </c>
       <c r="L15" t="n">
-        <v>98.33319308141191</v>
+        <v>88.08770683072242</v>
       </c>
     </row>
     <row r="16">
@@ -2398,37 +2398,37 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>117.7147641782954</v>
+        <v>107.0465007317839</v>
       </c>
       <c r="C16" t="n">
-        <v>108.3129151342385</v>
+        <v>97.08871625814072</v>
       </c>
       <c r="D16" t="n">
-        <v>105.2931235299014</v>
+        <v>94.10569447489254</v>
       </c>
       <c r="E16" t="n">
-        <v>103.5403782639467</v>
+        <v>92.31453327618252</v>
       </c>
       <c r="F16" t="n">
-        <v>102.3767925626486</v>
+        <v>91.05658796398694</v>
       </c>
       <c r="G16" t="n">
-        <v>101.3285394887185</v>
+        <v>90.102218220879</v>
       </c>
       <c r="H16" t="n">
-        <v>100.6060409812738</v>
+        <v>89.3153481221232</v>
       </c>
       <c r="I16" t="n">
-        <v>99.89998564744641</v>
+        <v>88.65053230274523</v>
       </c>
       <c r="J16" t="n">
-        <v>99.26285915944217</v>
+        <v>88.10436353522086</v>
       </c>
       <c r="K16" t="n">
-        <v>98.81319933569534</v>
+        <v>88.0855585222814</v>
       </c>
       <c r="L16" t="n">
-        <v>98.33319308141191</v>
+        <v>88.09441934855201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
resolve quality compare file
</commit_message>
<xml_diff>
--- a/quality_result.xlsx
+++ b/quality_result.xlsx
@@ -496,37 +496,37 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.0850703586590912</v>
+        <v>0.1294950434056319</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8376371584424092</v>
+        <v>1.26491607992532</v>
       </c>
       <c r="D2" t="n">
-        <v>1.664284004585596</v>
+        <v>2.513928729350673</v>
       </c>
       <c r="E2" t="n">
-        <v>2.517625568475289</v>
+        <v>3.785281012256375</v>
       </c>
       <c r="F2" t="n">
-        <v>3.367084493379861</v>
+        <v>3.35447914435808</v>
       </c>
       <c r="G2" t="n">
-        <v>4.191526726212222</v>
+        <v>4.219755854823064</v>
       </c>
       <c r="H2" t="n">
-        <v>5.027392635331763</v>
+        <v>5.040496856851308</v>
       </c>
       <c r="I2" t="n">
-        <v>5.901832978495572</v>
+        <v>5.882261051411582</v>
       </c>
       <c r="J2" t="n">
-        <v>6.664221015633858</v>
+        <v>5.047300323322493</v>
       </c>
       <c r="K2" t="n">
-        <v>6.666145957998967</v>
+        <v>5.654519239672482</v>
       </c>
       <c r="L2" t="n">
-        <v>6.67339472656496</v>
+        <v>6.303696382983146</v>
       </c>
     </row>
     <row r="3">
@@ -536,37 +536,37 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0821375930661762</v>
+        <v>0.1238487208849685</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8415248365436703</v>
+        <v>1.264273593426985</v>
       </c>
       <c r="D3" t="n">
-        <v>1.685579309389133</v>
+        <v>2.520958287508928</v>
       </c>
       <c r="E3" t="n">
-        <v>2.526804318522531</v>
+        <v>3.773973249885675</v>
       </c>
       <c r="F3" t="n">
-        <v>3.376192695801156</v>
+        <v>3.35514934680457</v>
       </c>
       <c r="G3" t="n">
-        <v>4.207027047455877</v>
+        <v>4.177843006336689</v>
       </c>
       <c r="H3" t="n">
-        <v>5.034785018707718</v>
+        <v>5.024832764333136</v>
       </c>
       <c r="I3" t="n">
-        <v>5.889240227264138</v>
+        <v>5.885816147847668</v>
       </c>
       <c r="J3" t="n">
-        <v>6.659307877398304</v>
+        <v>5.03072980935122</v>
       </c>
       <c r="K3" t="n">
-        <v>6.676518978571159</v>
+        <v>5.673793871045158</v>
       </c>
       <c r="L3" t="n">
-        <v>6.667546832285617</v>
+        <v>6.315446349441508</v>
       </c>
     </row>
     <row r="4">
@@ -576,37 +576,37 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0841406417314403</v>
+        <v>0.1262674935845833</v>
       </c>
       <c r="C4" t="n">
-        <v>0.8427493417654544</v>
+        <v>1.260966677626731</v>
       </c>
       <c r="D4" t="n">
-        <v>1.353302510739616</v>
+        <v>2.506921847186476</v>
       </c>
       <c r="E4" t="n">
-        <v>1.201617556280628</v>
+        <v>0.797930437608892</v>
       </c>
       <c r="F4" t="n">
-        <v>1.711674372315096</v>
+        <v>2.364723667468726</v>
       </c>
       <c r="G4" t="n">
-        <v>4.184431650688469</v>
+        <v>4.184101588581362</v>
       </c>
       <c r="H4" t="n">
-        <v>5.034996661585557</v>
+        <v>3.725161566661208</v>
       </c>
       <c r="I4" t="n">
-        <v>4.57409894304539</v>
+        <v>3.562330087302687</v>
       </c>
       <c r="J4" t="n">
-        <v>4.709512591491452</v>
+        <v>4.562894822871806</v>
       </c>
       <c r="K4" t="n">
-        <v>4.357220423537711</v>
+        <v>4.671093532983241</v>
       </c>
       <c r="L4" t="n">
-        <v>1.702551052545384</v>
+        <v>3.340269051177926</v>
       </c>
     </row>
     <row r="5">
@@ -616,37 +616,37 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0873304022474458</v>
+        <v>0.1260180576499356</v>
       </c>
       <c r="C5" t="n">
-        <v>0.8379672205495157</v>
+        <v>1.26723281065167</v>
       </c>
       <c r="D5" t="n">
-        <v>1.684054976757077</v>
+        <v>2.517016443875025</v>
       </c>
       <c r="E5" t="n">
-        <v>2.522961992466521</v>
+        <v>3.786815421187693</v>
       </c>
       <c r="F5" t="n">
-        <v>3.336965696216883</v>
+        <v>3.358895929653939</v>
       </c>
       <c r="G5" t="n">
-        <v>4.207092555965684</v>
+        <v>4.210627495937213</v>
       </c>
       <c r="H5" t="n">
-        <v>5.036014563045642</v>
+        <v>5.026750148024036</v>
       </c>
       <c r="I5" t="n">
-        <v>5.895375351163405</v>
+        <v>5.896423487320324</v>
       </c>
       <c r="J5" t="n">
-        <v>6.673535821816853</v>
+        <v>5.042698977499702</v>
       </c>
       <c r="K5" t="n">
-        <v>6.660645762733217</v>
+        <v>5.674145349617247</v>
       </c>
       <c r="L5" t="n">
-        <v>6.673150329432217</v>
+        <v>6.284582373538576</v>
       </c>
     </row>
     <row r="6">
@@ -656,37 +656,37 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.08590685193817005</v>
+        <v>0.1280966904386671</v>
       </c>
       <c r="C6" t="n">
-        <v>0.8414971214049056</v>
+        <v>1.268510224983654</v>
       </c>
       <c r="D6" t="n">
-        <v>1.684362362841558</v>
+        <v>2.520561457612898</v>
       </c>
       <c r="E6" t="n">
-        <v>2.523312211038184</v>
+        <v>3.781021704705647</v>
       </c>
       <c r="F6" t="n">
-        <v>3.362957457261996</v>
+        <v>3.359916350672092</v>
       </c>
       <c r="G6" t="n">
-        <v>4.190919512717469</v>
+        <v>4.215147583113922</v>
       </c>
       <c r="H6" t="n">
-        <v>5.049045717381171</v>
+        <v>5.035739931216065</v>
       </c>
       <c r="I6" t="n">
-        <v>5.883928998853601</v>
+        <v>5.895791078244875</v>
       </c>
       <c r="J6" t="n">
-        <v>6.664452814976253</v>
+        <v>5.044936346474727</v>
       </c>
       <c r="K6" t="n">
-        <v>6.650156842489827</v>
+        <v>5.687437286585423</v>
       </c>
       <c r="L6" t="n">
-        <v>6.669018254198214</v>
+        <v>6.30997953487669</v>
       </c>
     </row>
     <row r="7">
@@ -696,37 +696,37 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.08655941747817433</v>
+        <v>0.1255002891189242</v>
       </c>
       <c r="C7" t="n">
-        <v>0.8423058995452197</v>
+        <v>1.255169181812341</v>
       </c>
       <c r="D7" t="n">
-        <v>1.683523350004409</v>
+        <v>2.528773946794559</v>
       </c>
       <c r="E7" t="n">
-        <v>2.525761221481752</v>
+        <v>3.765208978181914</v>
       </c>
       <c r="F7" t="n">
-        <v>3.360833469809395</v>
+        <v>3.354121367112208</v>
       </c>
       <c r="G7" t="n">
-        <v>4.20550523438189</v>
+        <v>4.213192406051978</v>
       </c>
       <c r="H7" t="n">
-        <v>5.035954093651974</v>
+        <v>5.055135489235188</v>
       </c>
       <c r="I7" t="n">
-        <v>5.890119553030399</v>
+        <v>5.856359994456972</v>
       </c>
       <c r="J7" t="n">
-        <v>6.67049219566888</v>
+        <v>5.035588150258979</v>
       </c>
       <c r="K7" t="n">
-        <v>6.6599528842641</v>
+        <v>5.67970853733893</v>
       </c>
       <c r="L7" t="n">
-        <v>6.663114929641341</v>
+        <v>6.314274754201208</v>
       </c>
     </row>
     <row r="8">
@@ -736,37 +736,37 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.08343516547197621</v>
+        <v>0.1225902032147001</v>
       </c>
       <c r="C8" t="n">
-        <v>0.8420438655059902</v>
+        <v>1.263668900252082</v>
       </c>
       <c r="D8" t="n">
-        <v>1.681895715491503</v>
+        <v>2.514155489291262</v>
       </c>
       <c r="E8" t="n">
-        <v>2.507796772446113</v>
+        <v>3.789374029184005</v>
       </c>
       <c r="F8" t="n">
-        <v>3.357147356353696</v>
+        <v>3.357739452500032</v>
       </c>
       <c r="G8" t="n">
-        <v>4.198243868025548</v>
+        <v>4.196744730974187</v>
       </c>
       <c r="H8" t="n">
-        <v>5.042555335794102</v>
+        <v>5.042691391929855</v>
       </c>
       <c r="I8" t="n">
-        <v>5.866483578780282</v>
+        <v>5.878955391224379</v>
       </c>
       <c r="J8" t="n">
-        <v>6.646616863402159</v>
+        <v>5.049212669101821</v>
       </c>
       <c r="K8" t="n">
-        <v>6.674145554869676</v>
+        <v>5.671698227300815</v>
       </c>
       <c r="L8" t="n">
-        <v>6.673571095629827</v>
+        <v>6.293741602780083</v>
       </c>
     </row>
     <row r="9">
@@ -776,37 +776,37 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.08295644943876844</v>
+        <v>0.1264715775311133</v>
       </c>
       <c r="C9" t="n">
-        <v>0.8411670592977991</v>
+        <v>1.271813361451566</v>
       </c>
       <c r="D9" t="n">
-        <v>1.670970911702087</v>
+        <v>2.52112835746437</v>
       </c>
       <c r="E9" t="n">
-        <v>2.519142342433137</v>
+        <v>3.791777684554247</v>
       </c>
       <c r="F9" t="n">
-        <v>3.358865694957105</v>
+        <v>3.370120560853626</v>
       </c>
       <c r="G9" t="n">
-        <v>4.192972952544124</v>
+        <v>4.210705602237367</v>
       </c>
       <c r="H9" t="n">
-        <v>5.044694440595119</v>
+        <v>5.05227075171015</v>
       </c>
       <c r="I9" t="n">
-        <v>5.875443127275476</v>
+        <v>5.881354010506557</v>
       </c>
       <c r="J9" t="n">
-        <v>6.659267564469192</v>
+        <v>5.03918986078803</v>
       </c>
       <c r="K9" t="n">
-        <v>6.670421648042933</v>
+        <v>5.66836673954493</v>
       </c>
       <c r="L9" t="n">
-        <v>6.664336915305055</v>
+        <v>6.283524158482822</v>
       </c>
     </row>
     <row r="10">
@@ -816,37 +816,37 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.08421118935738671</v>
+        <v>0.1282818777234814</v>
       </c>
       <c r="C10" t="n">
-        <v>0.8440821879842275</v>
+        <v>1.259167715431392</v>
       </c>
       <c r="D10" t="n">
-        <v>1.667410776149863</v>
+        <v>2.025729694592153</v>
       </c>
       <c r="E10" t="n">
-        <v>2.518522531148037</v>
+        <v>2.305060148074241</v>
       </c>
       <c r="F10" t="n">
-        <v>3.368064601468902</v>
+        <v>1.380344927499717</v>
       </c>
       <c r="G10" t="n">
-        <v>4.209869108958289</v>
+        <v>2.555333274543645</v>
       </c>
       <c r="H10" t="n">
-        <v>4.708832310812683</v>
+        <v>5.025145189533756</v>
       </c>
       <c r="I10" t="n">
-        <v>4.219788609077968</v>
+        <v>5.224938585772056</v>
       </c>
       <c r="J10" t="n">
-        <v>4.676566850174479</v>
+        <v>4.286402125500526</v>
       </c>
       <c r="K10" t="n">
-        <v>6.683352020055683</v>
+        <v>4.936548669389051</v>
       </c>
       <c r="L10" t="n">
-        <v>5.008851207498205</v>
+        <v>5.063037492937359</v>
       </c>
     </row>
     <row r="11">
@@ -856,37 +856,37 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.08573048287330402</v>
+        <v>0.1266227508248393</v>
       </c>
       <c r="C11" t="n">
-        <v>0.8453772408319581</v>
+        <v>1.265086149880762</v>
       </c>
       <c r="D11" t="n">
-        <v>1.676949823001046</v>
+        <v>2.523433750193691</v>
       </c>
       <c r="E11" t="n">
-        <v>2.534431020798952</v>
+        <v>3.775175077570796</v>
       </c>
       <c r="F11" t="n">
-        <v>3.357107043424584</v>
+        <v>3.353277315158921</v>
       </c>
       <c r="G11" t="n">
-        <v>4.191589715163961</v>
+        <v>4.207032086572015</v>
       </c>
       <c r="H11" t="n">
-        <v>5.03566434447398</v>
+        <v>5.056899179883849</v>
       </c>
       <c r="I11" t="n">
-        <v>5.862628654933925</v>
+        <v>5.872084556368813</v>
       </c>
       <c r="J11" t="n">
-        <v>6.654923846357349</v>
+        <v>5.03576011020554</v>
       </c>
       <c r="K11" t="n">
-        <v>6.679580241625619</v>
+        <v>5.679855931578838</v>
       </c>
       <c r="L11" t="n">
-        <v>6.655256428022525</v>
+        <v>6.283441013014156</v>
       </c>
     </row>
     <row r="12">
@@ -896,37 +896,37 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.08471006185515061</v>
+        <v>0.1269704494004089</v>
       </c>
       <c r="C12" t="n">
-        <v>0.8411922548784944</v>
+        <v>1.259863112582531</v>
       </c>
       <c r="D12" t="n">
-        <v>1.682288766550347</v>
+        <v>2.528380896230872</v>
       </c>
       <c r="E12" t="n">
-        <v>2.518200027715139</v>
+        <v>3.781051939364392</v>
       </c>
       <c r="F12" t="n">
-        <v>3.370558963957722</v>
+        <v>3.376419456027413</v>
       </c>
       <c r="G12" t="n">
-        <v>4.203779337104272</v>
+        <v>4.194167223069074</v>
       </c>
       <c r="H12" t="n">
-        <v>5.029541818365058</v>
+        <v>5.033190138449716</v>
       </c>
       <c r="I12" t="n">
-        <v>5.861026216001713</v>
+        <v>5.86332909207725</v>
       </c>
       <c r="J12" t="n">
-        <v>6.664596429786216</v>
+        <v>5.030826182508083</v>
       </c>
       <c r="K12" t="n">
-        <v>6.672454931405031</v>
+        <v>5.675638188713759</v>
       </c>
       <c r="L12" t="n">
-        <v>6.652081784854937</v>
+        <v>6.287201455801569</v>
       </c>
     </row>
     <row r="13">
@@ -936,37 +936,37 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.08656445659431336</v>
+        <v>0.1282743190587951</v>
       </c>
       <c r="C13" t="n">
-        <v>0.8373952808677358</v>
+        <v>1.269016655517636</v>
       </c>
       <c r="D13" t="n">
-        <v>1.67427909144736</v>
+        <v>2.509491793179817</v>
       </c>
       <c r="E13" t="n">
-        <v>2.528772093374822</v>
+        <v>3.793236506838702</v>
       </c>
       <c r="F13" t="n">
-        <v>3.352458458786329</v>
+        <v>3.359787853210547</v>
       </c>
       <c r="G13" t="n">
-        <v>4.200904521346955</v>
+        <v>4.201652830093602</v>
       </c>
       <c r="H13" t="n">
-        <v>5.040862192771388</v>
+        <v>5.031794303279205</v>
       </c>
       <c r="I13" t="n">
-        <v>5.890552917018355</v>
+        <v>5.868252308545081</v>
       </c>
       <c r="J13" t="n">
-        <v>6.663049421131533</v>
+        <v>5.03768190433358</v>
       </c>
       <c r="K13" t="n">
-        <v>6.65616346892755</v>
+        <v>5.676222096664166</v>
       </c>
       <c r="L13" t="n">
-        <v>6.659335592537069</v>
+        <v>6.303715279680571</v>
       </c>
     </row>
     <row r="14">
@@ -976,37 +976,37 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.08489398959422517</v>
+        <v>0.1235690502915755</v>
       </c>
       <c r="C14" t="n">
-        <v>0.8385593166958516</v>
+        <v>1.254999111856899</v>
       </c>
       <c r="D14" t="n">
-        <v>1.684553849254841</v>
+        <v>2.525516162314765</v>
       </c>
       <c r="E14" t="n">
-        <v>2.532997392257398</v>
+        <v>3.783104116826721</v>
       </c>
       <c r="F14" t="n">
-        <v>3.363012887539526</v>
+        <v>3.372141246425377</v>
       </c>
       <c r="G14" t="n">
-        <v>4.199150908930574</v>
+        <v>4.20731931619194</v>
       </c>
       <c r="H14" t="n">
-        <v>5.048541805767268</v>
+        <v>5.047654921326799</v>
       </c>
       <c r="I14" t="n">
-        <v>5.881590848965091</v>
+        <v>5.871638594590509</v>
       </c>
       <c r="J14" t="n">
-        <v>6.689499741745298</v>
+        <v>5.042041372429341</v>
       </c>
       <c r="K14" t="n">
-        <v>6.656508648383074</v>
+        <v>5.671212582177013</v>
       </c>
       <c r="L14" t="n">
-        <v>6.660708751684955</v>
+        <v>6.290173906306395</v>
       </c>
     </row>
     <row r="15">
@@ -1016,37 +1016,37 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.08512074982048148</v>
+        <v>0.1291095515066308</v>
       </c>
       <c r="C15" t="n">
-        <v>0.8384963277441136</v>
+        <v>1.258986307478921</v>
       </c>
       <c r="D15" t="n">
-        <v>1.684478262512755</v>
+        <v>2.503917277973673</v>
       </c>
       <c r="E15" t="n">
-        <v>2.526925257309868</v>
+        <v>3.781456327925109</v>
       </c>
       <c r="F15" t="n">
-        <v>3.357462301112385</v>
+        <v>3.354418674964411</v>
       </c>
       <c r="G15" t="n">
-        <v>4.201655349651671</v>
+        <v>4.203225034328979</v>
       </c>
       <c r="H15" t="n">
-        <v>5.048466219025183</v>
+        <v>5.038423260560098</v>
       </c>
       <c r="I15" t="n">
-        <v>5.881815089633278</v>
+        <v>5.845382279948097</v>
       </c>
       <c r="J15" t="n">
-        <v>6.673334257171292</v>
+        <v>5.034977786932178</v>
       </c>
       <c r="K15" t="n">
-        <v>6.66535229720707</v>
+        <v>5.665621049409195</v>
       </c>
       <c r="L15" t="n">
-        <v>6.670769347056527</v>
+        <v>6.295922281662834</v>
       </c>
     </row>
     <row r="16">
@@ -1056,37 +1056,37 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.08478060948109702</v>
+        <v>0.1280777937769514</v>
       </c>
       <c r="C16" t="n">
-        <v>0.8396049332947001</v>
+        <v>1.26777325517674</v>
       </c>
       <c r="D16" t="n">
-        <v>1.668695750765316</v>
+        <v>2.525742922255354</v>
       </c>
       <c r="E16" t="n">
-        <v>2.520538177603648</v>
+        <v>3.784978665668923</v>
       </c>
       <c r="F16" t="n">
-        <v>3.367346527419091</v>
+        <v>3.361352498771716</v>
       </c>
       <c r="G16" t="n">
-        <v>4.194930649164137</v>
+        <v>4.220254727320828</v>
       </c>
       <c r="H16" t="n">
-        <v>5.028191335239799</v>
+        <v>5.047085501203089</v>
       </c>
       <c r="I16" t="n">
-        <v>5.859942806031822</v>
+        <v>5.881233071719221</v>
       </c>
       <c r="J16" t="n">
-        <v>6.645233626021995</v>
+        <v>5.049295814570487</v>
       </c>
       <c r="K16" t="n">
-        <v>6.674069968127591</v>
+        <v>5.67625611071953</v>
       </c>
       <c r="L16" t="n">
-        <v>6.660466874110281</v>
+        <v>6.289333003271018</v>
       </c>
     </row>
   </sheetData>
@@ -1167,37 +1167,37 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>101.002449283477</v>
+        <v>99.17813900922627</v>
       </c>
       <c r="C2" t="n">
-        <v>91.06967257308328</v>
+        <v>89.28005332992397</v>
       </c>
       <c r="D2" t="n">
-        <v>88.08795752952348</v>
+        <v>86.29714085318383</v>
       </c>
       <c r="E2" t="n">
-        <v>86.29032051623656</v>
+        <v>84.51968920209852</v>
       </c>
       <c r="F2" t="n">
-        <v>85.02769177474745</v>
+        <v>85.04398096052475</v>
       </c>
       <c r="G2" t="n">
-        <v>84.07650952481842</v>
+        <v>84.04735867726153</v>
       </c>
       <c r="H2" t="n">
-        <v>83.28680387551285</v>
+        <v>83.27549843892893</v>
       </c>
       <c r="I2" t="n">
-        <v>82.59036277323398</v>
+        <v>82.60478897812847</v>
       </c>
       <c r="J2" t="n">
-        <v>82.06273800352682</v>
+        <v>83.27004639629243</v>
       </c>
       <c r="K2" t="n">
-        <v>82.06148373670189</v>
+        <v>82.7766810031585</v>
       </c>
       <c r="L2" t="n">
-        <v>82.0567637833345</v>
+        <v>82.30468499196517</v>
       </c>
     </row>
     <row r="3">
@@ -1207,37 +1207,37 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>101.1748056611722</v>
+        <v>99.39131023237448</v>
       </c>
       <c r="C3" t="n">
-        <v>91.06955600239758</v>
+        <v>89.30181481739632</v>
       </c>
       <c r="D3" t="n">
-        <v>88.05273346758538</v>
+        <v>86.30456888993793</v>
       </c>
       <c r="E3" t="n">
-        <v>86.29450927925363</v>
+        <v>84.55223731231524</v>
       </c>
       <c r="F3" t="n">
-        <v>85.03595312426867</v>
+        <v>85.06310681832865</v>
       </c>
       <c r="G3" t="n">
-        <v>84.08047234239729</v>
+        <v>84.11070422224159</v>
       </c>
       <c r="H3" t="n">
-        <v>83.30041607135762</v>
+        <v>83.30900926179636</v>
       </c>
       <c r="I3" t="n">
-        <v>82.61963268461295</v>
+        <v>82.62215846247884</v>
       </c>
       <c r="J3" t="n">
-        <v>82.08593444456284</v>
+        <v>83.30391548193472</v>
       </c>
       <c r="K3" t="n">
-        <v>82.07472450535532</v>
+        <v>82.78148987213115</v>
       </c>
       <c r="L3" t="n">
-        <v>82.08056463573995</v>
+        <v>82.31618490938189</v>
       </c>
     </row>
     <row r="4">
@@ -1247,37 +1247,37 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>100.2952374680846</v>
+        <v>98.53040941833298</v>
       </c>
       <c r="C4" t="n">
-        <v>90.28831144833649</v>
+        <v>88.53628891586204</v>
       </c>
       <c r="D4" t="n">
-        <v>88.23134679267397</v>
+        <v>85.55191706500501</v>
       </c>
       <c r="E4" t="n">
-        <v>88.74763301835343</v>
+        <v>90.52367469768873</v>
       </c>
       <c r="F4" t="n">
-        <v>87.2110841848518</v>
+        <v>85.80749168765803</v>
       </c>
       <c r="G4" t="n">
-        <v>83.32893088415524</v>
+        <v>83.32927346307028</v>
       </c>
       <c r="H4" t="n">
-        <v>82.52530379884186</v>
+        <v>83.83384453227329</v>
       </c>
       <c r="I4" t="n">
-        <v>82.94224012154626</v>
+        <v>84.02795407880916</v>
       </c>
       <c r="J4" t="n">
-        <v>82.81553604440928</v>
+        <v>82.95246172084397</v>
       </c>
       <c r="K4" t="n">
-        <v>83.15320036190747</v>
+        <v>82.85068066660783</v>
       </c>
       <c r="L4" t="n">
-        <v>87.23429423322395</v>
+        <v>84.30705180589329</v>
       </c>
     </row>
     <row r="5">
@@ -1287,37 +1287,37 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>100.9143890595644</v>
+        <v>99.32171717247898</v>
       </c>
       <c r="C5" t="n">
-        <v>91.09377336188474</v>
+        <v>89.29748089722898</v>
       </c>
       <c r="D5" t="n">
-        <v>88.0624810135769</v>
+        <v>86.31718445842331</v>
       </c>
       <c r="E5" t="n">
-        <v>86.30693658424363</v>
+        <v>84.5433036163913</v>
       </c>
       <c r="F5" t="n">
-        <v>85.09252624338217</v>
+        <v>85.06407818410059</v>
       </c>
       <c r="G5" t="n">
-        <v>84.08622299904451</v>
+        <v>84.08257544363931</v>
       </c>
       <c r="H5" t="n">
-        <v>83.30517389176177</v>
+        <v>83.31317067112462</v>
       </c>
       <c r="I5" t="n">
-        <v>82.62092905200852</v>
+        <v>82.62015699041442</v>
       </c>
       <c r="J5" t="n">
-        <v>82.08248370507262</v>
+        <v>83.29938010318074</v>
       </c>
       <c r="K5" t="n">
-        <v>82.09088029580408</v>
+        <v>82.78700597619638</v>
       </c>
       <c r="L5" t="n">
-        <v>82.0827345796547</v>
+        <v>82.3432463115433</v>
       </c>
     </row>
     <row r="6">
@@ -1327,37 +1327,37 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>100.9801474610366</v>
+        <v>99.24504610280194</v>
       </c>
       <c r="C6" t="n">
-        <v>91.06989916004068</v>
+        <v>89.28748547294038</v>
       </c>
       <c r="D6" t="n">
-        <v>88.05607022157538</v>
+        <v>86.30545228457851</v>
       </c>
       <c r="E6" t="n">
-        <v>86.30071561305996</v>
+        <v>84.54433349141802</v>
       </c>
       <c r="F6" t="n">
-        <v>85.05321177330062</v>
+        <v>85.05714085463902</v>
       </c>
       <c r="G6" t="n">
-        <v>84.09733230464352</v>
+        <v>84.07229765693776</v>
       </c>
       <c r="H6" t="n">
-        <v>83.28833247581784</v>
+        <v>83.29979257633636</v>
       </c>
       <c r="I6" t="n">
-        <v>82.62375127210797</v>
+        <v>82.61500465108281</v>
       </c>
       <c r="J6" t="n">
-        <v>82.08278053225956</v>
+        <v>83.29186896328014</v>
       </c>
       <c r="K6" t="n">
-        <v>82.09210662519041</v>
+        <v>82.7712596643174</v>
       </c>
       <c r="L6" t="n">
-        <v>82.07980644527389</v>
+        <v>82.3201463660603</v>
       </c>
     </row>
     <row r="7">
@@ -1367,37 +1367,37 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>100.9709066973388</v>
+        <v>99.3575377843466</v>
       </c>
       <c r="C7" t="n">
-        <v>91.08935152301382</v>
+        <v>89.35696237279706</v>
       </c>
       <c r="D7" t="n">
-        <v>88.08185850509486</v>
+        <v>86.31488496302825</v>
       </c>
       <c r="E7" t="n">
-        <v>86.32012703665819</v>
+        <v>84.58609419153436</v>
       </c>
       <c r="F7" t="n">
-        <v>85.07958001224276</v>
+        <v>85.0882622154891</v>
       </c>
       <c r="G7" t="n">
-        <v>84.10586816963516</v>
+        <v>84.09793702087988</v>
       </c>
       <c r="H7" t="n">
-        <v>83.3232323227309</v>
+        <v>83.30672194647961</v>
       </c>
       <c r="I7" t="n">
-        <v>82.64280884974428</v>
+        <v>82.66777229570089</v>
       </c>
       <c r="J7" t="n">
-        <v>82.1024711443022</v>
+        <v>83.32354753434993</v>
       </c>
       <c r="K7" t="n">
-        <v>82.10933838048587</v>
+        <v>82.80078906509642</v>
       </c>
       <c r="L7" t="n">
-        <v>82.10727690500015</v>
+        <v>82.34081480824302</v>
       </c>
     </row>
     <row r="8">
@@ -1407,37 +1407,37 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>101.1301104831033</v>
+        <v>99.45902235479609</v>
       </c>
       <c r="C8" t="n">
-        <v>91.09025463639162</v>
+        <v>89.32724703103075</v>
       </c>
       <c r="D8" t="n">
-        <v>88.0856111566448</v>
+        <v>86.33965867088318</v>
       </c>
       <c r="E8" t="n">
-        <v>86.35067840798538</v>
+        <v>84.55790526128135</v>
       </c>
       <c r="F8" t="n">
-        <v>85.0838977560803</v>
+        <v>85.08313186352815</v>
       </c>
       <c r="G8" t="n">
-        <v>84.11292517580387</v>
+        <v>84.11447626059277</v>
       </c>
       <c r="H8" t="n">
-        <v>83.31709507147899</v>
+        <v>83.31697789352474</v>
       </c>
       <c r="I8" t="n">
-        <v>82.65982320552195</v>
+        <v>82.65060015072878</v>
       </c>
       <c r="J8" t="n">
-        <v>82.11759534813568</v>
+        <v>83.31137595878226</v>
       </c>
       <c r="K8" t="n">
-        <v>82.09964506054241</v>
+        <v>82.80648143734729</v>
       </c>
       <c r="L8" t="n">
-        <v>82.10001888399796</v>
+        <v>82.35452350666404</v>
       </c>
     </row>
     <row r="9">
@@ -1447,37 +1447,37 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>101.0938757052084</v>
+        <v>99.26244804656534</v>
       </c>
       <c r="C9" t="n">
-        <v>91.03355469298357</v>
+        <v>89.23814357084859</v>
       </c>
       <c r="D9" t="n">
-        <v>88.05268836612444</v>
+        <v>86.26642783033077</v>
       </c>
       <c r="E9" t="n">
-        <v>86.2698501865666</v>
+        <v>84.49394874055446</v>
       </c>
       <c r="F9" t="n">
-        <v>85.02045087543083</v>
+        <v>85.00592289000862</v>
       </c>
       <c r="G9" t="n">
-        <v>84.0571566543865</v>
+        <v>84.03882848228641</v>
       </c>
       <c r="H9" t="n">
-        <v>83.2540286040586</v>
+        <v>83.24751109970896</v>
       </c>
       <c r="I9" t="n">
-        <v>82.59197099594884</v>
+        <v>82.58760405118208</v>
       </c>
       <c r="J9" t="n">
-        <v>82.04811261488138</v>
+        <v>83.25876968353541</v>
       </c>
       <c r="K9" t="n">
-        <v>82.0408443912939</v>
+        <v>82.74779748816974</v>
       </c>
       <c r="L9" t="n">
-        <v>82.04480781668741</v>
+        <v>82.30034400697404</v>
       </c>
     </row>
     <row r="10">
@@ -1487,37 +1487,37 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>100.6307429408494</v>
+        <v>98.80237857484232</v>
       </c>
       <c r="C10" t="n">
-        <v>90.62059359459155</v>
+        <v>88.88319585747381</v>
       </c>
       <c r="D10" t="n">
-        <v>87.66401491313431</v>
+        <v>86.81821671422469</v>
       </c>
       <c r="E10" t="n">
-        <v>85.87298254757485</v>
+        <v>86.25720903441564</v>
       </c>
       <c r="F10" t="n">
-        <v>84.61063682311604</v>
+        <v>88.48456471602159</v>
       </c>
       <c r="G10" t="n">
-        <v>83.64175502054458</v>
+        <v>85.80996545036842</v>
       </c>
       <c r="H10" t="n">
-        <v>83.15530870459533</v>
+        <v>82.87295481071237</v>
       </c>
       <c r="I10" t="n">
-        <v>83.63153399782277</v>
+        <v>82.70362905153014</v>
       </c>
       <c r="J10" t="n">
-        <v>83.18516948403656</v>
+        <v>83.5636086344426</v>
       </c>
       <c r="K10" t="n">
-        <v>81.63449758713683</v>
+        <v>82.95030351985723</v>
       </c>
       <c r="L10" t="n">
-        <v>82.88705964477124</v>
+        <v>82.84042631614707</v>
       </c>
     </row>
     <row r="11">
@@ -1527,37 +1527,37 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>101.0074308147476</v>
+        <v>99.31358083156503</v>
       </c>
       <c r="C11" t="n">
-        <v>91.06827799739176</v>
+        <v>89.31749726185755</v>
       </c>
       <c r="D11" t="n">
-        <v>88.09358283332958</v>
+        <v>86.31877919980491</v>
       </c>
       <c r="E11" t="n">
-        <v>86.29997875756328</v>
+        <v>84.5693273002635</v>
       </c>
       <c r="F11" t="n">
-        <v>85.07913162137926</v>
+        <v>85.08408880399257</v>
       </c>
       <c r="G11" t="n">
-        <v>84.11499585288388</v>
+        <v>84.09902527007628</v>
       </c>
       <c r="H11" t="n">
-        <v>83.3182157713799</v>
+        <v>83.29994056225429</v>
       </c>
       <c r="I11" t="n">
-        <v>82.65785964966963</v>
+        <v>82.65086050681971</v>
       </c>
       <c r="J11" t="n">
-        <v>82.10735261234274</v>
+        <v>83.3181106480319</v>
       </c>
       <c r="K11" t="n">
-        <v>82.09129179966925</v>
+        <v>82.79538778077104</v>
       </c>
       <c r="L11" t="n">
-        <v>82.10713557789389</v>
+        <v>82.3567855571948</v>
       </c>
     </row>
     <row r="12">
@@ -1567,37 +1567,37 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>101.0364449555497</v>
+        <v>99.27876861699693</v>
       </c>
       <c r="C12" t="n">
-        <v>91.06684229070513</v>
+        <v>89.31256157986708</v>
       </c>
       <c r="D12" t="n">
-        <v>88.05678949474287</v>
+        <v>86.28737018182632</v>
       </c>
       <c r="E12" t="n">
-        <v>86.30489270042447</v>
+        <v>84.53966875239783</v>
       </c>
       <c r="F12" t="n">
-        <v>85.03877565405878</v>
+        <v>85.03123100266443</v>
       </c>
       <c r="G12" t="n">
-        <v>84.07939583253662</v>
+        <v>84.0893375245394</v>
       </c>
       <c r="H12" t="n">
-        <v>83.30051070955724</v>
+        <v>83.29736157400001</v>
       </c>
       <c r="I12" t="n">
-        <v>82.63605830459525</v>
+        <v>82.63435223827656</v>
       </c>
       <c r="J12" t="n">
-        <v>82.07805638285438</v>
+        <v>83.29940180669749</v>
       </c>
       <c r="K12" t="n">
-        <v>82.07293845357358</v>
+        <v>82.77564790959666</v>
       </c>
       <c r="L12" t="n">
-        <v>82.08621914349041</v>
+        <v>82.3312211684288</v>
       </c>
     </row>
     <row r="13">
@@ -1607,37 +1607,37 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>100.9579956542617</v>
+        <v>99.2500618915316</v>
       </c>
       <c r="C13" t="n">
-        <v>91.10208663428818</v>
+        <v>89.2967858490903</v>
       </c>
       <c r="D13" t="n">
-        <v>88.09311318768556</v>
+        <v>86.33560127302556</v>
       </c>
       <c r="E13" t="n">
-        <v>86.30229482389697</v>
+        <v>84.54135985403607</v>
       </c>
       <c r="F13" t="n">
-        <v>85.07775767431613</v>
+        <v>85.06827316891722</v>
       </c>
       <c r="G13" t="n">
-        <v>84.09796361574962</v>
+        <v>84.09719007420341</v>
       </c>
       <c r="H13" t="n">
-        <v>83.30634347682957</v>
+        <v>83.31416293425747</v>
       </c>
       <c r="I13" t="n">
-        <v>82.62983110757168</v>
+        <v>82.64630394240264</v>
       </c>
       <c r="J13" t="n">
-        <v>82.09466138002361</v>
+        <v>83.30914904736888</v>
       </c>
       <c r="K13" t="n">
-        <v>82.09915193263504</v>
+        <v>82.79086265997674</v>
       </c>
       <c r="L13" t="n">
-        <v>82.09708271119734</v>
+        <v>82.33549056877365</v>
       </c>
     </row>
     <row r="14">
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>101.0125463363493</v>
+        <v>99.38188993228145</v>
       </c>
       <c r="C14" t="n">
-        <v>91.06597788899977</v>
+        <v>89.3145528360803</v>
       </c>
       <c r="D14" t="n">
-        <v>88.03646678967296</v>
+        <v>86.27748549909901</v>
       </c>
       <c r="E14" t="n">
-        <v>86.26496834690789</v>
+        <v>84.52250408174473</v>
       </c>
       <c r="F14" t="n">
-        <v>85.03403045776155</v>
+        <v>85.02225820061186</v>
       </c>
       <c r="G14" t="n">
-        <v>84.06970094794181</v>
+        <v>84.06126103149407</v>
       </c>
       <c r="H14" t="n">
-        <v>83.26965620472305</v>
+        <v>83.27041920296878</v>
       </c>
       <c r="I14" t="n">
-        <v>82.60636767710155</v>
+        <v>82.61372260914158</v>
       </c>
       <c r="J14" t="n">
-        <v>82.04737936064672</v>
+        <v>83.27521884899011</v>
       </c>
       <c r="K14" t="n">
-        <v>82.06885076777432</v>
+        <v>82.76452362981206</v>
       </c>
       <c r="L14" t="n">
-        <v>82.06611133401256</v>
+        <v>82.31465637174091</v>
       </c>
     </row>
     <row r="15">
@@ -1687,37 +1687,37 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>100.9546778215397</v>
+        <v>99.14580566002067</v>
       </c>
       <c r="C15" t="n">
-        <v>91.02002057858152</v>
+        <v>89.25517931681674</v>
       </c>
       <c r="D15" t="n">
-        <v>87.99037811815325</v>
+        <v>86.26918961532952</v>
       </c>
       <c r="E15" t="n">
-        <v>86.22910826454871</v>
+        <v>84.47879849412246</v>
       </c>
       <c r="F15" t="n">
-        <v>84.99492077838617</v>
+        <v>84.99885955541859</v>
       </c>
       <c r="G15" t="n">
-        <v>84.02082797242988</v>
+        <v>84.01920580680594</v>
       </c>
       <c r="H15" t="n">
-        <v>83.22343768184109</v>
+        <v>83.23208574503921</v>
       </c>
       <c r="I15" t="n">
-        <v>82.55991855586574</v>
+        <v>82.58690304092596</v>
       </c>
       <c r="J15" t="n">
-        <v>82.01160344233861</v>
+        <v>83.23521139139929</v>
       </c>
       <c r="K15" t="n">
-        <v>82.01680113787914</v>
+        <v>82.72271175088967</v>
       </c>
       <c r="L15" t="n">
-        <v>82.01327298321775</v>
+        <v>82.26459339683279</v>
       </c>
     </row>
     <row r="16">
@@ -1727,37 +1727,37 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>100.9790000906037</v>
+        <v>99.18685580149113</v>
       </c>
       <c r="C16" t="n">
-        <v>91.0212156169605</v>
+        <v>89.23117832422955</v>
       </c>
       <c r="D16" t="n">
-        <v>88.03819383371234</v>
+        <v>86.23770273456294</v>
       </c>
       <c r="E16" t="n">
-        <v>86.24703263500228</v>
+        <v>84.48095982212868</v>
       </c>
       <c r="F16" t="n">
-        <v>84.98908732280671</v>
+        <v>84.99682484901908</v>
       </c>
       <c r="G16" t="n">
-        <v>84.03471757969879</v>
+        <v>84.00857878391291</v>
       </c>
       <c r="H16" t="n">
-        <v>83.24784748094297</v>
+        <v>83.23155881360351</v>
       </c>
       <c r="I16" t="n">
-        <v>82.58303166156502</v>
+        <v>82.56728152693347</v>
       </c>
       <c r="J16" t="n">
-        <v>82.03686289404064</v>
+        <v>83.22937953773911</v>
       </c>
       <c r="K16" t="n">
-        <v>82.0180578811012</v>
+        <v>82.72106786047564</v>
       </c>
       <c r="L16" t="n">
-        <v>82.02691870737181</v>
+        <v>82.27564178430075</v>
       </c>
     </row>
   </sheetData>
@@ -1838,37 +1838,37 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>107.0316834372365</v>
+        <v>105.2069346199184</v>
       </c>
       <c r="C2" t="n">
-        <v>97.09890672684276</v>
+        <v>95.30884894061603</v>
       </c>
       <c r="D2" t="n">
-        <v>94.11719168328293</v>
+        <v>92.32593646387591</v>
       </c>
       <c r="E2" t="n">
-        <v>92.31955466999602</v>
+        <v>90.5484848127906</v>
       </c>
       <c r="F2" t="n">
-        <v>91.05692592850693</v>
+        <v>91.07321511428421</v>
       </c>
       <c r="G2" t="n">
-        <v>90.10574367857787</v>
+        <v>90.07659283102099</v>
       </c>
       <c r="H2" t="n">
-        <v>89.31603802927229</v>
+        <v>89.30473259268838</v>
       </c>
       <c r="I2" t="n">
-        <v>88.61959692699344</v>
+        <v>88.63402313188793</v>
       </c>
       <c r="J2" t="n">
-        <v>88.09197215728629</v>
+        <v>89.29887460735925</v>
       </c>
       <c r="K2" t="n">
-        <v>88.09071789046135</v>
+        <v>88.80550921422531</v>
       </c>
       <c r="L2" t="n">
-        <v>88.08599793709396</v>
+        <v>88.333513203032</v>
       </c>
     </row>
     <row r="3">
@@ -1878,37 +1878,37 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>107.1840463525335</v>
+        <v>105.4005508199797</v>
       </c>
       <c r="C3" t="n">
-        <v>97.07879669375886</v>
+        <v>95.31105540500158</v>
       </c>
       <c r="D3" t="n">
-        <v>94.06197415894668</v>
+        <v>92.31380947754317</v>
       </c>
       <c r="E3" t="n">
-        <v>92.3037499706149</v>
+        <v>90.56147789992052</v>
       </c>
       <c r="F3" t="n">
-        <v>91.04519381562996</v>
+        <v>91.07234750968996</v>
       </c>
       <c r="G3" t="n">
-        <v>90.08971303375857</v>
+        <v>90.11994491360289</v>
       </c>
       <c r="H3" t="n">
-        <v>89.3096567627189</v>
+        <v>89.31824995315763</v>
       </c>
       <c r="I3" t="n">
-        <v>88.62887337597425</v>
+        <v>88.63139915384012</v>
       </c>
       <c r="J3" t="n">
-        <v>88.09517513592412</v>
+        <v>89.31315614684752</v>
       </c>
       <c r="K3" t="n">
-        <v>88.0839651967166</v>
+        <v>88.79073053704391</v>
       </c>
       <c r="L3" t="n">
-        <v>88.08980532710123</v>
+        <v>88.32542557429468</v>
       </c>
     </row>
     <row r="4">
@@ -1918,37 +1918,37 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>107.0794078752054</v>
+        <v>105.3165504774222</v>
       </c>
       <c r="C4" t="n">
-        <v>97.07248185545726</v>
+        <v>95.32242997495123</v>
       </c>
       <c r="D4" t="n">
-        <v>95.01551719979476</v>
+        <v>92.33805812409422</v>
       </c>
       <c r="E4" t="n">
-        <v>95.53180342547419</v>
+        <v>97.30981575677795</v>
       </c>
       <c r="F4" t="n">
-        <v>93.99525459197258</v>
+        <v>92.59166209477881</v>
       </c>
       <c r="G4" t="n">
-        <v>90.11310129127601</v>
+        <v>90.11344387019105</v>
       </c>
       <c r="H4" t="n">
-        <v>89.30947420596266</v>
+        <v>90.61801493939406</v>
       </c>
       <c r="I4" t="n">
-        <v>89.72641052866705</v>
+        <v>90.81212448592993</v>
       </c>
       <c r="J4" t="n">
-        <v>89.59970645153005</v>
+        <v>89.73706149358944</v>
       </c>
       <c r="K4" t="n">
-        <v>89.93737076902823</v>
+        <v>89.63528043935329</v>
       </c>
       <c r="L4" t="n">
-        <v>94.01846464034472</v>
+        <v>91.09165157863876</v>
       </c>
     </row>
     <row r="5">
@@ -1958,37 +1958,37 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>106.9178114698907</v>
+        <v>105.3251382609694</v>
       </c>
       <c r="C5" t="n">
-        <v>97.09719577221107</v>
+        <v>95.30090198571938</v>
       </c>
       <c r="D5" t="n">
-        <v>94.06590342390322</v>
+        <v>92.32060554691371</v>
       </c>
       <c r="E5" t="n">
-        <v>92.31035899456997</v>
+        <v>90.5467247048817</v>
       </c>
       <c r="F5" t="n">
-        <v>91.09594865370849</v>
+        <v>91.0675005944269</v>
       </c>
       <c r="G5" t="n">
-        <v>90.08964540937083</v>
+        <v>90.08599785396562</v>
       </c>
       <c r="H5" t="n">
-        <v>89.30859630208808</v>
+        <v>89.31659308145093</v>
       </c>
       <c r="I5" t="n">
-        <v>88.62435146233483</v>
+        <v>88.62357940074074</v>
       </c>
       <c r="J5" t="n">
-        <v>88.08590611539893</v>
+        <v>89.30283563684819</v>
       </c>
       <c r="K5" t="n">
-        <v>88.09430270613041</v>
+        <v>88.79046150986385</v>
       </c>
       <c r="L5" t="n">
-        <v>88.08615698998102</v>
+        <v>88.34670184521076</v>
       </c>
     </row>
     <row r="6">
@@ -1998,37 +1998,37 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>106.9891880295116</v>
+        <v>105.2540869826038</v>
       </c>
       <c r="C6" t="n">
-        <v>97.07893972851578</v>
+        <v>95.29652635274221</v>
       </c>
       <c r="D6" t="n">
-        <v>94.0651107900505</v>
+        <v>92.31449316438037</v>
       </c>
       <c r="E6" t="n">
-        <v>92.30975618153505</v>
+        <v>90.55337437121986</v>
       </c>
       <c r="F6" t="n">
-        <v>91.06225234177572</v>
+        <v>91.0661814231141</v>
       </c>
       <c r="G6" t="n">
-        <v>90.10637287311859</v>
+        <v>90.08133822541284</v>
       </c>
       <c r="H6" t="n">
-        <v>89.29737304429293</v>
+        <v>89.30883314481144</v>
       </c>
       <c r="I6" t="n">
-        <v>88.63279184058305</v>
+        <v>88.6240452195579</v>
       </c>
       <c r="J6" t="n">
-        <v>88.09182110073468</v>
+        <v>89.30090916551063</v>
       </c>
       <c r="K6" t="n">
-        <v>88.10114719366551</v>
+        <v>88.78029986654789</v>
       </c>
       <c r="L6" t="n">
-        <v>88.08884701374899</v>
+        <v>88.32918656829079</v>
       </c>
     </row>
     <row r="7">
@@ -2038,37 +2038,37 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>106.9563228244436</v>
+        <v>105.3430188121457</v>
       </c>
       <c r="C7" t="n">
-        <v>97.07476765011864</v>
+        <v>95.3424434005961</v>
       </c>
       <c r="D7" t="n">
-        <v>94.06727463219968</v>
+        <v>92.30036599082732</v>
       </c>
       <c r="E7" t="n">
-        <v>92.30554316376302</v>
+        <v>90.57157521933341</v>
       </c>
       <c r="F7" t="n">
-        <v>91.0649961393476</v>
+        <v>91.07367834259394</v>
       </c>
       <c r="G7" t="n">
-        <v>90.09128429674</v>
+        <v>90.08335314798472</v>
       </c>
       <c r="H7" t="n">
-        <v>89.30864844983574</v>
+        <v>89.29213807358445</v>
       </c>
       <c r="I7" t="n">
-        <v>88.62822497684914</v>
+        <v>88.65318842280573</v>
       </c>
       <c r="J7" t="n">
-        <v>88.08788727140706</v>
+        <v>89.30896404637991</v>
       </c>
       <c r="K7" t="n">
-        <v>88.09475450759069</v>
+        <v>88.78620557712644</v>
       </c>
       <c r="L7" t="n">
-        <v>88.09269303210499</v>
+        <v>88.32623132027305</v>
       </c>
     </row>
     <row r="8">
@@ -2078,37 +2078,37 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>107.1159747593838</v>
+        <v>105.4449084256669</v>
       </c>
       <c r="C8" t="n">
-        <v>97.07611891267217</v>
+        <v>95.3131331019015</v>
       </c>
       <c r="D8" t="n">
-        <v>94.07147543292535</v>
+        <v>92.32554474175393</v>
       </c>
       <c r="E8" t="n">
-        <v>92.33654268426592</v>
+        <v>90.54379133215208</v>
       </c>
       <c r="F8" t="n">
-        <v>91.06976203236087</v>
+        <v>91.0689961398087</v>
       </c>
       <c r="G8" t="n">
-        <v>90.09878945208443</v>
+        <v>90.10034053687333</v>
       </c>
       <c r="H8" t="n">
-        <v>89.30295934775954</v>
+        <v>89.30284216980527</v>
       </c>
       <c r="I8" t="n">
-        <v>88.64568748180248</v>
+        <v>88.63646442700933</v>
       </c>
       <c r="J8" t="n">
-        <v>88.10345962441623</v>
+        <v>89.29722944287522</v>
       </c>
       <c r="K8" t="n">
-        <v>88.08550933682297</v>
+        <v>88.79233492144024</v>
       </c>
       <c r="L8" t="n">
-        <v>88.08588316027851</v>
+        <v>88.34037699075697</v>
       </c>
     </row>
     <row r="9">
@@ -2118,37 +2118,37 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>107.1409645168747</v>
+        <v>105.3095367180777</v>
       </c>
       <c r="C9" t="n">
-        <v>97.08064350464987</v>
+        <v>95.28523224236102</v>
       </c>
       <c r="D9" t="n">
-        <v>94.09977717779074</v>
+        <v>92.31351650184317</v>
       </c>
       <c r="E9" t="n">
-        <v>92.3169389982329</v>
+        <v>90.5410374120669</v>
       </c>
       <c r="F9" t="n">
-        <v>91.06753968709712</v>
+        <v>91.05301170167492</v>
       </c>
       <c r="G9" t="n">
-        <v>90.1042454660528</v>
+        <v>90.0859172939527</v>
       </c>
       <c r="H9" t="n">
-        <v>89.30111741572492</v>
+        <v>89.29459991137526</v>
       </c>
       <c r="I9" t="n">
-        <v>88.63905980761515</v>
+        <v>88.6346928628484</v>
       </c>
       <c r="J9" t="n">
-        <v>88.09520142654767</v>
+        <v>89.30585886019497</v>
       </c>
       <c r="K9" t="n">
-        <v>88.08793320296019</v>
+        <v>88.79488666482931</v>
       </c>
       <c r="L9" t="n">
-        <v>88.09189662835372</v>
+        <v>88.34743318363363</v>
       </c>
     </row>
     <row r="10">
@@ -2158,37 +2158,37 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>107.0757680637159</v>
+        <v>105.2478129925057</v>
       </c>
       <c r="C10" t="n">
-        <v>97.06561871745807</v>
+        <v>95.32863027513714</v>
       </c>
       <c r="D10" t="n">
-        <v>94.10904003600082</v>
+        <v>93.26365113188805</v>
       </c>
       <c r="E10" t="n">
-        <v>92.31800767044136</v>
+        <v>92.702643452079</v>
       </c>
       <c r="F10" t="n">
-        <v>91.05566194598255</v>
+        <v>94.92958983888811</v>
       </c>
       <c r="G10" t="n">
-        <v>90.08678014341112</v>
+        <v>92.25499057323495</v>
       </c>
       <c r="H10" t="n">
-        <v>89.60033382746187</v>
+        <v>89.3179799335789</v>
       </c>
       <c r="I10" t="n">
-        <v>90.07655912068928</v>
+        <v>89.14865417439668</v>
       </c>
       <c r="J10" t="n">
-        <v>89.63019460690307</v>
+        <v>90.00853695912474</v>
       </c>
       <c r="K10" t="n">
-        <v>88.07952271000335</v>
+        <v>89.39523184453934</v>
       </c>
       <c r="L10" t="n">
-        <v>89.33208476763775</v>
+        <v>89.2853546408292</v>
       </c>
     </row>
     <row r="11">
@@ -2198,37 +2198,37 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>106.9981133765165</v>
+        <v>105.304348633816</v>
       </c>
       <c r="C11" t="n">
-        <v>97.05896055916068</v>
+        <v>95.30826506410853</v>
       </c>
       <c r="D11" t="n">
-        <v>94.0842653950985</v>
+        <v>92.30954700205589</v>
       </c>
       <c r="E11" t="n">
-        <v>92.2906613193322</v>
+        <v>90.56009510251445</v>
       </c>
       <c r="F11" t="n">
-        <v>91.06981418314818</v>
+        <v>91.07477136576149</v>
       </c>
       <c r="G11" t="n">
-        <v>90.10567841465281</v>
+        <v>90.0897078318452</v>
       </c>
       <c r="H11" t="n">
-        <v>89.30889833314882</v>
+        <v>89.29062312402321</v>
       </c>
       <c r="I11" t="n">
-        <v>88.64854221143855</v>
+        <v>88.64154306858863</v>
       </c>
       <c r="J11" t="n">
-        <v>88.09803517411167</v>
+        <v>89.3088157419941</v>
       </c>
       <c r="K11" t="n">
-        <v>88.08197436143817</v>
+        <v>88.78609287473324</v>
       </c>
       <c r="L11" t="n">
-        <v>88.09781813966282</v>
+        <v>88.34749065115699</v>
       </c>
     </row>
     <row r="12">
@@ -2238,37 +2238,37 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>107.0501160866807</v>
+        <v>105.2924395079227</v>
       </c>
       <c r="C12" t="n">
-        <v>97.08051342183614</v>
+        <v>95.32623247079286</v>
       </c>
       <c r="D12" t="n">
-        <v>94.07046062587389</v>
+        <v>92.30104107275208</v>
       </c>
       <c r="E12" t="n">
-        <v>92.31856383155548</v>
+        <v>90.5533396433236</v>
       </c>
       <c r="F12" t="n">
-        <v>91.05244678518979</v>
+        <v>91.04490213379543</v>
       </c>
       <c r="G12" t="n">
-        <v>90.09306696366762</v>
+        <v>90.10300865567041</v>
       </c>
       <c r="H12" t="n">
-        <v>89.31418184068825</v>
+        <v>89.31103270513103</v>
       </c>
       <c r="I12" t="n">
-        <v>88.64972943572626</v>
+        <v>88.64802336940757</v>
       </c>
       <c r="J12" t="n">
-        <v>88.0917275139854</v>
+        <v>89.31307295031158</v>
       </c>
       <c r="K12" t="n">
-        <v>88.0866095847046</v>
+        <v>88.78931905321075</v>
       </c>
       <c r="L12" t="n">
-        <v>88.09989027462143</v>
+        <v>88.34489231204289</v>
       </c>
     </row>
     <row r="13">
@@ -2278,37 +2278,37 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>106.9560700042771</v>
+        <v>105.24806889639</v>
       </c>
       <c r="C13" t="n">
-        <v>97.10016098430359</v>
+        <v>95.29479285394868</v>
       </c>
       <c r="D13" t="n">
-        <v>94.09118753770096</v>
+        <v>92.33360827788394</v>
       </c>
       <c r="E13" t="n">
-        <v>92.30036917391239</v>
+        <v>90.53936685889443</v>
       </c>
       <c r="F13" t="n">
-        <v>91.07583202433155</v>
+        <v>91.06634751893264</v>
       </c>
       <c r="G13" t="n">
-        <v>90.09603796576505</v>
+        <v>90.09526442421884</v>
       </c>
       <c r="H13" t="n">
-        <v>89.30441782684497</v>
+        <v>89.3122372842729</v>
       </c>
       <c r="I13" t="n">
-        <v>88.62790545758708</v>
+        <v>88.64437829241805</v>
       </c>
       <c r="J13" t="n">
-        <v>88.09273573003904</v>
+        <v>89.30715866272749</v>
       </c>
       <c r="K13" t="n">
-        <v>88.09722628265047</v>
+        <v>88.78887227533532</v>
       </c>
       <c r="L13" t="n">
-        <v>88.09515706121275</v>
+        <v>88.33350018413226</v>
       </c>
     </row>
     <row r="14">
@@ -2318,37 +2318,37 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>107.0406966379376</v>
+        <v>105.4103689867681</v>
       </c>
       <c r="C14" t="n">
-        <v>97.09412819058812</v>
+        <v>95.34303189056695</v>
       </c>
       <c r="D14" t="n">
-        <v>94.06461709126131</v>
+        <v>92.30596455358567</v>
       </c>
       <c r="E14" t="n">
-        <v>92.29311864849626</v>
+        <v>90.55098313623141</v>
       </c>
       <c r="F14" t="n">
-        <v>91.06218075934989</v>
+        <v>91.05040850220021</v>
       </c>
       <c r="G14" t="n">
-        <v>90.09785124953018</v>
+        <v>90.08941133308242</v>
       </c>
       <c r="H14" t="n">
-        <v>89.29780650631137</v>
+        <v>89.29856950455714</v>
       </c>
       <c r="I14" t="n">
-        <v>88.63451797868991</v>
+        <v>88.64187291072993</v>
       </c>
       <c r="J14" t="n">
-        <v>88.07552966223506</v>
+        <v>89.30340202575623</v>
       </c>
       <c r="K14" t="n">
-        <v>88.09700106936268</v>
+        <v>88.7927068065782</v>
       </c>
       <c r="L14" t="n">
-        <v>88.09426163560093</v>
+        <v>88.34283954850703</v>
       </c>
     </row>
     <row r="15">
@@ -2358,37 +2358,37 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>107.0291116690444</v>
+        <v>105.2198823503031</v>
       </c>
       <c r="C15" t="n">
-        <v>97.0944544260862</v>
+        <v>95.32925600709916</v>
       </c>
       <c r="D15" t="n">
-        <v>94.06481196565792</v>
+        <v>92.34326630561196</v>
       </c>
       <c r="E15" t="n">
-        <v>92.30354211205339</v>
+        <v>90.55287518440487</v>
       </c>
       <c r="F15" t="n">
-        <v>91.06935462589085</v>
+        <v>91.07329340292327</v>
       </c>
       <c r="G15" t="n">
-        <v>90.09526181993456</v>
+        <v>90.09363965431064</v>
       </c>
       <c r="H15" t="n">
-        <v>89.29787152934574</v>
+        <v>89.30651959254388</v>
       </c>
       <c r="I15" t="n">
-        <v>88.63435240337041</v>
+        <v>88.66133688843064</v>
       </c>
       <c r="J15" t="n">
-        <v>88.08603728984329</v>
+        <v>89.30949048635709</v>
       </c>
       <c r="K15" t="n">
-        <v>88.09123498538382</v>
+        <v>88.79699084584749</v>
       </c>
       <c r="L15" t="n">
-        <v>88.08770683072242</v>
+        <v>88.33887249179062</v>
       </c>
     </row>
     <row r="16">
@@ -2398,37 +2398,37 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>107.0465007317839</v>
+        <v>105.2547276955889</v>
       </c>
       <c r="C16" t="n">
-        <v>97.08871625814072</v>
+        <v>95.29905021832731</v>
       </c>
       <c r="D16" t="n">
-        <v>94.10569447489254</v>
+        <v>92.30557462866068</v>
       </c>
       <c r="E16" t="n">
-        <v>92.31453327618252</v>
+        <v>90.54883171622643</v>
       </c>
       <c r="F16" t="n">
-        <v>91.05658796398694</v>
+        <v>91.06432549019928</v>
       </c>
       <c r="G16" t="n">
-        <v>90.102218220879</v>
+        <v>90.07607942509311</v>
       </c>
       <c r="H16" t="n">
-        <v>89.3153481221232</v>
+        <v>89.29905945478373</v>
       </c>
       <c r="I16" t="n">
-        <v>88.65053230274523</v>
+        <v>88.63478216811367</v>
       </c>
       <c r="J16" t="n">
-        <v>88.10436353522086</v>
+        <v>89.29715792811976</v>
       </c>
       <c r="K16" t="n">
-        <v>88.0855585222814</v>
+        <v>88.7888462508563</v>
       </c>
       <c r="L16" t="n">
-        <v>88.09441934855201</v>
+        <v>88.34342017468143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>